<commit_message>
Sync current local repository to staging
</commit_message>
<xml_diff>
--- a/5_BATCH_EXPORT/cars24-batch-processing-template.xlsx
+++ b/5_BATCH_EXPORT/cars24-batch-processing-template.xlsx
@@ -118,7 +118,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>One row equals one post/request.</t>
+          <t>One row equals one generated output request. Number of slides defaults to 1; use a higher value for carousel rows.</t>
         </is>
       </c>
     </row>
@@ -135,7 +135,7 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>Validation warnings should be blank before upload.</t>
+          <t>Validation warnings should be blank before upload; slide counts must be between 1 and 10.</t>
         </is>
       </c>
     </row>
@@ -193,66 +193,49 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>Slides per post</t>
+          <t>Default dimensions</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Default 1</t>
+          <t>1000 x 650 px</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>Use 1 for a single image; use 2-10 for a carousel in that row.</t>
+          <t>Matches the current Autonauts blog-cover batch.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>Default dimensions</t>
+          <t>Default theme</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>1000 x 650 px</t>
+          <t>Dark Cars24 brand blue</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>Matches the current Autonauts blog-cover batch.</t>
+          <t>Can be changed row by row.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Default theme</t>
+          <t>Default visible text</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>Dark Cars24 brand blue</t>
+          <t>Blog title only</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t>Can be changed row by row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="0" t="inlineStr">
-        <is>
-          <t>Default visible text</t>
-        </is>
-      </c>
-      <c r="B12" s="0" t="inlineStr">
-        <is>
-          <t>Blog title only</t>
-        </is>
-      </c>
-      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Description remains prompt context only.</t>
         </is>
@@ -271,8 +254,8 @@
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="4" width="36" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="52" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
     <col min="7" max="8" width="14" customWidth="1"/>
     <col min="9" max="13" width="20" customWidth="1"/>
     <col min="14" max="18" width="34" customWidth="1"/>
@@ -303,12 +286,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Slides per post</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>Number of slides</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -404,10 +387,10 @@
       <c r="B2" s="0"/>
       <c r="C2" s="0"/>
       <c r="D2" s="0"/>
-      <c r="E2" s="0">
-        <v>1</v>
-      </c>
-      <c r="F2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0">
+        <v>1</v>
+      </c>
       <c r="G2" s="0">
         <v>1000</v>
       </c>
@@ -449,7 +432,7 @@
       </c>
       <c r="V2" s="0"/>
       <c r="W2" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C2="","Missing blog title",""),IF(E2="","Missing slides per post",""),IF(OR(E2&lt;1,E2&gt;10),"Slides per post must be 1-10",""),IF(F2="","Missing URL",""),IF(G2="","Missing width",""),IF(H2="","Missing height",""),IF(I2="","Missing theme",""),IF(M2="","Missing hero type",""),IF(N2="","Missing image direction",""),IF(U2="","Missing status",""),IF(AND(J2="Custom",K2=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C2="","Missing blog title",""),IF(E2="","Missing URL",""),IF(F2="","Missing number of slides",""),IF(OR(F2&lt;1,F2&gt;10),"Number of slides must be 1-10",""),IF(G2="","Missing width",""),IF(H2="","Missing height",""),IF(I2="","Missing theme",""),IF(M2="","Missing hero type",""),IF(N2="","Missing image direction",""),IF(U2="","Missing status",""),IF(AND(J2="Custom",K2=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="3">
@@ -459,10 +442,10 @@
       <c r="B3" s="0"/>
       <c r="C3" s="0"/>
       <c r="D3" s="0"/>
-      <c r="E3" s="0">
-        <v>1</v>
-      </c>
-      <c r="F3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0">
+        <v>1</v>
+      </c>
       <c r="G3" s="0">
         <v>1000</v>
       </c>
@@ -504,7 +487,7 @@
       </c>
       <c r="V3" s="0"/>
       <c r="W3" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C3="","Missing blog title",""),IF(E3="","Missing slides per post",""),IF(OR(E3&lt;1,E3&gt;10),"Slides per post must be 1-10",""),IF(F3="","Missing URL",""),IF(G3="","Missing width",""),IF(H3="","Missing height",""),IF(I3="","Missing theme",""),IF(M3="","Missing hero type",""),IF(N3="","Missing image direction",""),IF(U3="","Missing status",""),IF(AND(J3="Custom",K3=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C3="","Missing blog title",""),IF(E3="","Missing URL",""),IF(F3="","Missing number of slides",""),IF(OR(F3&lt;1,F3&gt;10),"Number of slides must be 1-10",""),IF(G3="","Missing width",""),IF(H3="","Missing height",""),IF(I3="","Missing theme",""),IF(M3="","Missing hero type",""),IF(N3="","Missing image direction",""),IF(U3="","Missing status",""),IF(AND(J3="Custom",K3=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="4">
@@ -514,10 +497,10 @@
       <c r="B4" s="0"/>
       <c r="C4" s="0"/>
       <c r="D4" s="0"/>
-      <c r="E4" s="0">
-        <v>1</v>
-      </c>
-      <c r="F4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0">
+        <v>1</v>
+      </c>
       <c r="G4" s="0">
         <v>1000</v>
       </c>
@@ -559,7 +542,7 @@
       </c>
       <c r="V4" s="0"/>
       <c r="W4" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C4="","Missing blog title",""),IF(E4="","Missing slides per post",""),IF(OR(E4&lt;1,E4&gt;10),"Slides per post must be 1-10",""),IF(F4="","Missing URL",""),IF(G4="","Missing width",""),IF(H4="","Missing height",""),IF(I4="","Missing theme",""),IF(M4="","Missing hero type",""),IF(N4="","Missing image direction",""),IF(U4="","Missing status",""),IF(AND(J4="Custom",K4=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C4="","Missing blog title",""),IF(E4="","Missing URL",""),IF(F4="","Missing number of slides",""),IF(OR(F4&lt;1,F4&gt;10),"Number of slides must be 1-10",""),IF(G4="","Missing width",""),IF(H4="","Missing height",""),IF(I4="","Missing theme",""),IF(M4="","Missing hero type",""),IF(N4="","Missing image direction",""),IF(U4="","Missing status",""),IF(AND(J4="Custom",K4=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="5">
@@ -569,10 +552,10 @@
       <c r="B5" s="0"/>
       <c r="C5" s="0"/>
       <c r="D5" s="0"/>
-      <c r="E5" s="0">
-        <v>1</v>
-      </c>
-      <c r="F5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0">
+        <v>1</v>
+      </c>
       <c r="G5" s="0">
         <v>1000</v>
       </c>
@@ -614,7 +597,7 @@
       </c>
       <c r="V5" s="0"/>
       <c r="W5" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C5="","Missing blog title",""),IF(E5="","Missing slides per post",""),IF(OR(E5&lt;1,E5&gt;10),"Slides per post must be 1-10",""),IF(F5="","Missing URL",""),IF(G5="","Missing width",""),IF(H5="","Missing height",""),IF(I5="","Missing theme",""),IF(M5="","Missing hero type",""),IF(N5="","Missing image direction",""),IF(U5="","Missing status",""),IF(AND(J5="Custom",K5=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C5="","Missing blog title",""),IF(E5="","Missing URL",""),IF(F5="","Missing number of slides",""),IF(OR(F5&lt;1,F5&gt;10),"Number of slides must be 1-10",""),IF(G5="","Missing width",""),IF(H5="","Missing height",""),IF(I5="","Missing theme",""),IF(M5="","Missing hero type",""),IF(N5="","Missing image direction",""),IF(U5="","Missing status",""),IF(AND(J5="Custom",K5=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="6">
@@ -624,10 +607,10 @@
       <c r="B6" s="0"/>
       <c r="C6" s="0"/>
       <c r="D6" s="0"/>
-      <c r="E6" s="0">
-        <v>1</v>
-      </c>
-      <c r="F6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0">
+        <v>1</v>
+      </c>
       <c r="G6" s="0">
         <v>1000</v>
       </c>
@@ -669,7 +652,7 @@
       </c>
       <c r="V6" s="0"/>
       <c r="W6" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C6="","Missing blog title",""),IF(E6="","Missing slides per post",""),IF(OR(E6&lt;1,E6&gt;10),"Slides per post must be 1-10",""),IF(F6="","Missing URL",""),IF(G6="","Missing width",""),IF(H6="","Missing height",""),IF(I6="","Missing theme",""),IF(M6="","Missing hero type",""),IF(N6="","Missing image direction",""),IF(U6="","Missing status",""),IF(AND(J6="Custom",K6=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C6="","Missing blog title",""),IF(E6="","Missing URL",""),IF(F6="","Missing number of slides",""),IF(OR(F6&lt;1,F6&gt;10),"Number of slides must be 1-10",""),IF(G6="","Missing width",""),IF(H6="","Missing height",""),IF(I6="","Missing theme",""),IF(M6="","Missing hero type",""),IF(N6="","Missing image direction",""),IF(U6="","Missing status",""),IF(AND(J6="Custom",K6=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="7">
@@ -679,10 +662,10 @@
       <c r="B7" s="0"/>
       <c r="C7" s="0"/>
       <c r="D7" s="0"/>
-      <c r="E7" s="0">
-        <v>1</v>
-      </c>
-      <c r="F7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0">
+        <v>1</v>
+      </c>
       <c r="G7" s="0">
         <v>1000</v>
       </c>
@@ -724,7 +707,7 @@
       </c>
       <c r="V7" s="0"/>
       <c r="W7" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C7="","Missing blog title",""),IF(E7="","Missing slides per post",""),IF(OR(E7&lt;1,E7&gt;10),"Slides per post must be 1-10",""),IF(F7="","Missing URL",""),IF(G7="","Missing width",""),IF(H7="","Missing height",""),IF(I7="","Missing theme",""),IF(M7="","Missing hero type",""),IF(N7="","Missing image direction",""),IF(U7="","Missing status",""),IF(AND(J7="Custom",K7=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C7="","Missing blog title",""),IF(E7="","Missing URL",""),IF(F7="","Missing number of slides",""),IF(OR(F7&lt;1,F7&gt;10),"Number of slides must be 1-10",""),IF(G7="","Missing width",""),IF(H7="","Missing height",""),IF(I7="","Missing theme",""),IF(M7="","Missing hero type",""),IF(N7="","Missing image direction",""),IF(U7="","Missing status",""),IF(AND(J7="Custom",K7=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="8">
@@ -734,10 +717,10 @@
       <c r="B8" s="0"/>
       <c r="C8" s="0"/>
       <c r="D8" s="0"/>
-      <c r="E8" s="0">
-        <v>1</v>
-      </c>
-      <c r="F8" s="0"/>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0">
+        <v>1</v>
+      </c>
       <c r="G8" s="0">
         <v>1000</v>
       </c>
@@ -779,7 +762,7 @@
       </c>
       <c r="V8" s="0"/>
       <c r="W8" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C8="","Missing blog title",""),IF(E8="","Missing slides per post",""),IF(OR(E8&lt;1,E8&gt;10),"Slides per post must be 1-10",""),IF(F8="","Missing URL",""),IF(G8="","Missing width",""),IF(H8="","Missing height",""),IF(I8="","Missing theme",""),IF(M8="","Missing hero type",""),IF(N8="","Missing image direction",""),IF(U8="","Missing status",""),IF(AND(J8="Custom",K8=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C8="","Missing blog title",""),IF(E8="","Missing URL",""),IF(F8="","Missing number of slides",""),IF(OR(F8&lt;1,F8&gt;10),"Number of slides must be 1-10",""),IF(G8="","Missing width",""),IF(H8="","Missing height",""),IF(I8="","Missing theme",""),IF(M8="","Missing hero type",""),IF(N8="","Missing image direction",""),IF(U8="","Missing status",""),IF(AND(J8="Custom",K8=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="9">
@@ -789,10 +772,10 @@
       <c r="B9" s="0"/>
       <c r="C9" s="0"/>
       <c r="D9" s="0"/>
-      <c r="E9" s="0">
-        <v>1</v>
-      </c>
-      <c r="F9" s="0"/>
+      <c r="E9" s="0"/>
+      <c r="F9" s="0">
+        <v>1</v>
+      </c>
       <c r="G9" s="0">
         <v>1000</v>
       </c>
@@ -834,7 +817,7 @@
       </c>
       <c r="V9" s="0"/>
       <c r="W9" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C9="","Missing blog title",""),IF(E9="","Missing slides per post",""),IF(OR(E9&lt;1,E9&gt;10),"Slides per post must be 1-10",""),IF(F9="","Missing URL",""),IF(G9="","Missing width",""),IF(H9="","Missing height",""),IF(I9="","Missing theme",""),IF(M9="","Missing hero type",""),IF(N9="","Missing image direction",""),IF(U9="","Missing status",""),IF(AND(J9="Custom",K9=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C9="","Missing blog title",""),IF(E9="","Missing URL",""),IF(F9="","Missing number of slides",""),IF(OR(F9&lt;1,F9&gt;10),"Number of slides must be 1-10",""),IF(G9="","Missing width",""),IF(H9="","Missing height",""),IF(I9="","Missing theme",""),IF(M9="","Missing hero type",""),IF(N9="","Missing image direction",""),IF(U9="","Missing status",""),IF(AND(J9="Custom",K9=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="10">
@@ -844,10 +827,10 @@
       <c r="B10" s="0"/>
       <c r="C10" s="0"/>
       <c r="D10" s="0"/>
-      <c r="E10" s="0">
-        <v>1</v>
-      </c>
-      <c r="F10" s="0"/>
+      <c r="E10" s="0"/>
+      <c r="F10" s="0">
+        <v>1</v>
+      </c>
       <c r="G10" s="0">
         <v>1000</v>
       </c>
@@ -889,7 +872,7 @@
       </c>
       <c r="V10" s="0"/>
       <c r="W10" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C10="","Missing blog title",""),IF(E10="","Missing slides per post",""),IF(OR(E10&lt;1,E10&gt;10),"Slides per post must be 1-10",""),IF(F10="","Missing URL",""),IF(G10="","Missing width",""),IF(H10="","Missing height",""),IF(I10="","Missing theme",""),IF(M10="","Missing hero type",""),IF(N10="","Missing image direction",""),IF(U10="","Missing status",""),IF(AND(J10="Custom",K10=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C10="","Missing blog title",""),IF(E10="","Missing URL",""),IF(F10="","Missing number of slides",""),IF(OR(F10&lt;1,F10&gt;10),"Number of slides must be 1-10",""),IF(G10="","Missing width",""),IF(H10="","Missing height",""),IF(I10="","Missing theme",""),IF(M10="","Missing hero type",""),IF(N10="","Missing image direction",""),IF(U10="","Missing status",""),IF(AND(J10="Custom",K10=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="11">
@@ -899,10 +882,10 @@
       <c r="B11" s="0"/>
       <c r="C11" s="0"/>
       <c r="D11" s="0"/>
-      <c r="E11" s="0">
-        <v>1</v>
-      </c>
-      <c r="F11" s="0"/>
+      <c r="E11" s="0"/>
+      <c r="F11" s="0">
+        <v>1</v>
+      </c>
       <c r="G11" s="0">
         <v>1000</v>
       </c>
@@ -944,7 +927,7 @@
       </c>
       <c r="V11" s="0"/>
       <c r="W11" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C11="","Missing blog title",""),IF(E11="","Missing slides per post",""),IF(OR(E11&lt;1,E11&gt;10),"Slides per post must be 1-10",""),IF(F11="","Missing URL",""),IF(G11="","Missing width",""),IF(H11="","Missing height",""),IF(I11="","Missing theme",""),IF(M11="","Missing hero type",""),IF(N11="","Missing image direction",""),IF(U11="","Missing status",""),IF(AND(J11="Custom",K11=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C11="","Missing blog title",""),IF(E11="","Missing URL",""),IF(F11="","Missing number of slides",""),IF(OR(F11&lt;1,F11&gt;10),"Number of slides must be 1-10",""),IF(G11="","Missing width",""),IF(H11="","Missing height",""),IF(I11="","Missing theme",""),IF(M11="","Missing hero type",""),IF(N11="","Missing image direction",""),IF(U11="","Missing status",""),IF(AND(J11="Custom",K11=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="12">
@@ -954,10 +937,10 @@
       <c r="B12" s="0"/>
       <c r="C12" s="0"/>
       <c r="D12" s="0"/>
-      <c r="E12" s="0">
-        <v>1</v>
-      </c>
-      <c r="F12" s="0"/>
+      <c r="E12" s="0"/>
+      <c r="F12" s="0">
+        <v>1</v>
+      </c>
       <c r="G12" s="0">
         <v>1000</v>
       </c>
@@ -999,7 +982,7 @@
       </c>
       <c r="V12" s="0"/>
       <c r="W12" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C12="","Missing blog title",""),IF(E12="","Missing slides per post",""),IF(OR(E12&lt;1,E12&gt;10),"Slides per post must be 1-10",""),IF(F12="","Missing URL",""),IF(G12="","Missing width",""),IF(H12="","Missing height",""),IF(I12="","Missing theme",""),IF(M12="","Missing hero type",""),IF(N12="","Missing image direction",""),IF(U12="","Missing status",""),IF(AND(J12="Custom",K12=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C12="","Missing blog title",""),IF(E12="","Missing URL",""),IF(F12="","Missing number of slides",""),IF(OR(F12&lt;1,F12&gt;10),"Number of slides must be 1-10",""),IF(G12="","Missing width",""),IF(H12="","Missing height",""),IF(I12="","Missing theme",""),IF(M12="","Missing hero type",""),IF(N12="","Missing image direction",""),IF(U12="","Missing status",""),IF(AND(J12="Custom",K12=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="13">
@@ -1009,10 +992,10 @@
       <c r="B13" s="0"/>
       <c r="C13" s="0"/>
       <c r="D13" s="0"/>
-      <c r="E13" s="0">
-        <v>1</v>
-      </c>
-      <c r="F13" s="0"/>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0">
+        <v>1</v>
+      </c>
       <c r="G13" s="0">
         <v>1000</v>
       </c>
@@ -1054,7 +1037,7 @@
       </c>
       <c r="V13" s="0"/>
       <c r="W13" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C13="","Missing blog title",""),IF(E13="","Missing slides per post",""),IF(OR(E13&lt;1,E13&gt;10),"Slides per post must be 1-10",""),IF(F13="","Missing URL",""),IF(G13="","Missing width",""),IF(H13="","Missing height",""),IF(I13="","Missing theme",""),IF(M13="","Missing hero type",""),IF(N13="","Missing image direction",""),IF(U13="","Missing status",""),IF(AND(J13="Custom",K13=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C13="","Missing blog title",""),IF(E13="","Missing URL",""),IF(F13="","Missing number of slides",""),IF(OR(F13&lt;1,F13&gt;10),"Number of slides must be 1-10",""),IF(G13="","Missing width",""),IF(H13="","Missing height",""),IF(I13="","Missing theme",""),IF(M13="","Missing hero type",""),IF(N13="","Missing image direction",""),IF(U13="","Missing status",""),IF(AND(J13="Custom",K13=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="14">
@@ -1064,10 +1047,10 @@
       <c r="B14" s="0"/>
       <c r="C14" s="0"/>
       <c r="D14" s="0"/>
-      <c r="E14" s="0">
-        <v>1</v>
-      </c>
-      <c r="F14" s="0"/>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0">
+        <v>1</v>
+      </c>
       <c r="G14" s="0">
         <v>1000</v>
       </c>
@@ -1109,7 +1092,7 @@
       </c>
       <c r="V14" s="0"/>
       <c r="W14" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C14="","Missing blog title",""),IF(E14="","Missing slides per post",""),IF(OR(E14&lt;1,E14&gt;10),"Slides per post must be 1-10",""),IF(F14="","Missing URL",""),IF(G14="","Missing width",""),IF(H14="","Missing height",""),IF(I14="","Missing theme",""),IF(M14="","Missing hero type",""),IF(N14="","Missing image direction",""),IF(U14="","Missing status",""),IF(AND(J14="Custom",K14=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C14="","Missing blog title",""),IF(E14="","Missing URL",""),IF(F14="","Missing number of slides",""),IF(OR(F14&lt;1,F14&gt;10),"Number of slides must be 1-10",""),IF(G14="","Missing width",""),IF(H14="","Missing height",""),IF(I14="","Missing theme",""),IF(M14="","Missing hero type",""),IF(N14="","Missing image direction",""),IF(U14="","Missing status",""),IF(AND(J14="Custom",K14=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="15">
@@ -1119,10 +1102,10 @@
       <c r="B15" s="0"/>
       <c r="C15" s="0"/>
       <c r="D15" s="0"/>
-      <c r="E15" s="0">
-        <v>1</v>
-      </c>
-      <c r="F15" s="0"/>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0">
+        <v>1</v>
+      </c>
       <c r="G15" s="0">
         <v>1000</v>
       </c>
@@ -1164,7 +1147,7 @@
       </c>
       <c r="V15" s="0"/>
       <c r="W15" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C15="","Missing blog title",""),IF(E15="","Missing slides per post",""),IF(OR(E15&lt;1,E15&gt;10),"Slides per post must be 1-10",""),IF(F15="","Missing URL",""),IF(G15="","Missing width",""),IF(H15="","Missing height",""),IF(I15="","Missing theme",""),IF(M15="","Missing hero type",""),IF(N15="","Missing image direction",""),IF(U15="","Missing status",""),IF(AND(J15="Custom",K15=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C15="","Missing blog title",""),IF(E15="","Missing URL",""),IF(F15="","Missing number of slides",""),IF(OR(F15&lt;1,F15&gt;10),"Number of slides must be 1-10",""),IF(G15="","Missing width",""),IF(H15="","Missing height",""),IF(I15="","Missing theme",""),IF(M15="","Missing hero type",""),IF(N15="","Missing image direction",""),IF(U15="","Missing status",""),IF(AND(J15="Custom",K15=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="16">
@@ -1174,10 +1157,10 @@
       <c r="B16" s="0"/>
       <c r="C16" s="0"/>
       <c r="D16" s="0"/>
-      <c r="E16" s="0">
-        <v>1</v>
-      </c>
-      <c r="F16" s="0"/>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0">
+        <v>1</v>
+      </c>
       <c r="G16" s="0">
         <v>1000</v>
       </c>
@@ -1219,7 +1202,7 @@
       </c>
       <c r="V16" s="0"/>
       <c r="W16" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C16="","Missing blog title",""),IF(E16="","Missing slides per post",""),IF(OR(E16&lt;1,E16&gt;10),"Slides per post must be 1-10",""),IF(F16="","Missing URL",""),IF(G16="","Missing width",""),IF(H16="","Missing height",""),IF(I16="","Missing theme",""),IF(M16="","Missing hero type",""),IF(N16="","Missing image direction",""),IF(U16="","Missing status",""),IF(AND(J16="Custom",K16=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C16="","Missing blog title",""),IF(E16="","Missing URL",""),IF(F16="","Missing number of slides",""),IF(OR(F16&lt;1,F16&gt;10),"Number of slides must be 1-10",""),IF(G16="","Missing width",""),IF(H16="","Missing height",""),IF(I16="","Missing theme",""),IF(M16="","Missing hero type",""),IF(N16="","Missing image direction",""),IF(U16="","Missing status",""),IF(AND(J16="Custom",K16=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="17">
@@ -1229,10 +1212,10 @@
       <c r="B17" s="0"/>
       <c r="C17" s="0"/>
       <c r="D17" s="0"/>
-      <c r="E17" s="0">
-        <v>1</v>
-      </c>
-      <c r="F17" s="0"/>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0">
+        <v>1</v>
+      </c>
       <c r="G17" s="0">
         <v>1000</v>
       </c>
@@ -1274,7 +1257,7 @@
       </c>
       <c r="V17" s="0"/>
       <c r="W17" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C17="","Missing blog title",""),IF(E17="","Missing slides per post",""),IF(OR(E17&lt;1,E17&gt;10),"Slides per post must be 1-10",""),IF(F17="","Missing URL",""),IF(G17="","Missing width",""),IF(H17="","Missing height",""),IF(I17="","Missing theme",""),IF(M17="","Missing hero type",""),IF(N17="","Missing image direction",""),IF(U17="","Missing status",""),IF(AND(J17="Custom",K17=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C17="","Missing blog title",""),IF(E17="","Missing URL",""),IF(F17="","Missing number of slides",""),IF(OR(F17&lt;1,F17&gt;10),"Number of slides must be 1-10",""),IF(G17="","Missing width",""),IF(H17="","Missing height",""),IF(I17="","Missing theme",""),IF(M17="","Missing hero type",""),IF(N17="","Missing image direction",""),IF(U17="","Missing status",""),IF(AND(J17="Custom",K17=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="18">
@@ -1284,10 +1267,10 @@
       <c r="B18" s="0"/>
       <c r="C18" s="0"/>
       <c r="D18" s="0"/>
-      <c r="E18" s="0">
-        <v>1</v>
-      </c>
-      <c r="F18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0">
+        <v>1</v>
+      </c>
       <c r="G18" s="0">
         <v>1000</v>
       </c>
@@ -1329,7 +1312,7 @@
       </c>
       <c r="V18" s="0"/>
       <c r="W18" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C18="","Missing blog title",""),IF(E18="","Missing slides per post",""),IF(OR(E18&lt;1,E18&gt;10),"Slides per post must be 1-10",""),IF(F18="","Missing URL",""),IF(G18="","Missing width",""),IF(H18="","Missing height",""),IF(I18="","Missing theme",""),IF(M18="","Missing hero type",""),IF(N18="","Missing image direction",""),IF(U18="","Missing status",""),IF(AND(J18="Custom",K18=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C18="","Missing blog title",""),IF(E18="","Missing URL",""),IF(F18="","Missing number of slides",""),IF(OR(F18&lt;1,F18&gt;10),"Number of slides must be 1-10",""),IF(G18="","Missing width",""),IF(H18="","Missing height",""),IF(I18="","Missing theme",""),IF(M18="","Missing hero type",""),IF(N18="","Missing image direction",""),IF(U18="","Missing status",""),IF(AND(J18="Custom",K18=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="19">
@@ -1339,10 +1322,10 @@
       <c r="B19" s="0"/>
       <c r="C19" s="0"/>
       <c r="D19" s="0"/>
-      <c r="E19" s="0">
-        <v>1</v>
-      </c>
-      <c r="F19" s="0"/>
+      <c r="E19" s="0"/>
+      <c r="F19" s="0">
+        <v>1</v>
+      </c>
       <c r="G19" s="0">
         <v>1000</v>
       </c>
@@ -1384,7 +1367,7 @@
       </c>
       <c r="V19" s="0"/>
       <c r="W19" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C19="","Missing blog title",""),IF(E19="","Missing slides per post",""),IF(OR(E19&lt;1,E19&gt;10),"Slides per post must be 1-10",""),IF(F19="","Missing URL",""),IF(G19="","Missing width",""),IF(H19="","Missing height",""),IF(I19="","Missing theme",""),IF(M19="","Missing hero type",""),IF(N19="","Missing image direction",""),IF(U19="","Missing status",""),IF(AND(J19="Custom",K19=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C19="","Missing blog title",""),IF(E19="","Missing URL",""),IF(F19="","Missing number of slides",""),IF(OR(F19&lt;1,F19&gt;10),"Number of slides must be 1-10",""),IF(G19="","Missing width",""),IF(H19="","Missing height",""),IF(I19="","Missing theme",""),IF(M19="","Missing hero type",""),IF(N19="","Missing image direction",""),IF(U19="","Missing status",""),IF(AND(J19="Custom",K19=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="20">
@@ -1394,10 +1377,10 @@
       <c r="B20" s="0"/>
       <c r="C20" s="0"/>
       <c r="D20" s="0"/>
-      <c r="E20" s="0">
-        <v>1</v>
-      </c>
-      <c r="F20" s="0"/>
+      <c r="E20" s="0"/>
+      <c r="F20" s="0">
+        <v>1</v>
+      </c>
       <c r="G20" s="0">
         <v>1000</v>
       </c>
@@ -1439,7 +1422,7 @@
       </c>
       <c r="V20" s="0"/>
       <c r="W20" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C20="","Missing blog title",""),IF(E20="","Missing slides per post",""),IF(OR(E20&lt;1,E20&gt;10),"Slides per post must be 1-10",""),IF(F20="","Missing URL",""),IF(G20="","Missing width",""),IF(H20="","Missing height",""),IF(I20="","Missing theme",""),IF(M20="","Missing hero type",""),IF(N20="","Missing image direction",""),IF(U20="","Missing status",""),IF(AND(J20="Custom",K20=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C20="","Missing blog title",""),IF(E20="","Missing URL",""),IF(F20="","Missing number of slides",""),IF(OR(F20&lt;1,F20&gt;10),"Number of slides must be 1-10",""),IF(G20="","Missing width",""),IF(H20="","Missing height",""),IF(I20="","Missing theme",""),IF(M20="","Missing hero type",""),IF(N20="","Missing image direction",""),IF(U20="","Missing status",""),IF(AND(J20="Custom",K20=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="21">
@@ -1449,10 +1432,10 @@
       <c r="B21" s="0"/>
       <c r="C21" s="0"/>
       <c r="D21" s="0"/>
-      <c r="E21" s="0">
-        <v>1</v>
-      </c>
-      <c r="F21" s="0"/>
+      <c r="E21" s="0"/>
+      <c r="F21" s="0">
+        <v>1</v>
+      </c>
       <c r="G21" s="0">
         <v>1000</v>
       </c>
@@ -1494,7 +1477,7 @@
       </c>
       <c r="V21" s="0"/>
       <c r="W21" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C21="","Missing blog title",""),IF(E21="","Missing slides per post",""),IF(OR(E21&lt;1,E21&gt;10),"Slides per post must be 1-10",""),IF(F21="","Missing URL",""),IF(G21="","Missing width",""),IF(H21="","Missing height",""),IF(I21="","Missing theme",""),IF(M21="","Missing hero type",""),IF(N21="","Missing image direction",""),IF(U21="","Missing status",""),IF(AND(J21="Custom",K21=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C21="","Missing blog title",""),IF(E21="","Missing URL",""),IF(F21="","Missing number of slides",""),IF(OR(F21&lt;1,F21&gt;10),"Number of slides must be 1-10",""),IF(G21="","Missing width",""),IF(H21="","Missing height",""),IF(I21="","Missing theme",""),IF(M21="","Missing hero type",""),IF(N21="","Missing image direction",""),IF(U21="","Missing status",""),IF(AND(J21="Custom",K21=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="22">
@@ -1504,10 +1487,10 @@
       <c r="B22" s="0"/>
       <c r="C22" s="0"/>
       <c r="D22" s="0"/>
-      <c r="E22" s="0">
-        <v>1</v>
-      </c>
-      <c r="F22" s="0"/>
+      <c r="E22" s="0"/>
+      <c r="F22" s="0">
+        <v>1</v>
+      </c>
       <c r="G22" s="0">
         <v>1000</v>
       </c>
@@ -1549,7 +1532,7 @@
       </c>
       <c r="V22" s="0"/>
       <c r="W22" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C22="","Missing blog title",""),IF(E22="","Missing slides per post",""),IF(OR(E22&lt;1,E22&gt;10),"Slides per post must be 1-10",""),IF(F22="","Missing URL",""),IF(G22="","Missing width",""),IF(H22="","Missing height",""),IF(I22="","Missing theme",""),IF(M22="","Missing hero type",""),IF(N22="","Missing image direction",""),IF(U22="","Missing status",""),IF(AND(J22="Custom",K22=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C22="","Missing blog title",""),IF(E22="","Missing URL",""),IF(F22="","Missing number of slides",""),IF(OR(F22&lt;1,F22&gt;10),"Number of slides must be 1-10",""),IF(G22="","Missing width",""),IF(H22="","Missing height",""),IF(I22="","Missing theme",""),IF(M22="","Missing hero type",""),IF(N22="","Missing image direction",""),IF(U22="","Missing status",""),IF(AND(J22="Custom",K22=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="23">
@@ -1559,10 +1542,10 @@
       <c r="B23" s="0"/>
       <c r="C23" s="0"/>
       <c r="D23" s="0"/>
-      <c r="E23" s="0">
-        <v>1</v>
-      </c>
-      <c r="F23" s="0"/>
+      <c r="E23" s="0"/>
+      <c r="F23" s="0">
+        <v>1</v>
+      </c>
       <c r="G23" s="0">
         <v>1000</v>
       </c>
@@ -1604,7 +1587,7 @@
       </c>
       <c r="V23" s="0"/>
       <c r="W23" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C23="","Missing blog title",""),IF(E23="","Missing slides per post",""),IF(OR(E23&lt;1,E23&gt;10),"Slides per post must be 1-10",""),IF(F23="","Missing URL",""),IF(G23="","Missing width",""),IF(H23="","Missing height",""),IF(I23="","Missing theme",""),IF(M23="","Missing hero type",""),IF(N23="","Missing image direction",""),IF(U23="","Missing status",""),IF(AND(J23="Custom",K23=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C23="","Missing blog title",""),IF(E23="","Missing URL",""),IF(F23="","Missing number of slides",""),IF(OR(F23&lt;1,F23&gt;10),"Number of slides must be 1-10",""),IF(G23="","Missing width",""),IF(H23="","Missing height",""),IF(I23="","Missing theme",""),IF(M23="","Missing hero type",""),IF(N23="","Missing image direction",""),IF(U23="","Missing status",""),IF(AND(J23="Custom",K23=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="24">
@@ -1614,10 +1597,10 @@
       <c r="B24" s="0"/>
       <c r="C24" s="0"/>
       <c r="D24" s="0"/>
-      <c r="E24" s="0">
-        <v>1</v>
-      </c>
-      <c r="F24" s="0"/>
+      <c r="E24" s="0"/>
+      <c r="F24" s="0">
+        <v>1</v>
+      </c>
       <c r="G24" s="0">
         <v>1000</v>
       </c>
@@ -1659,7 +1642,7 @@
       </c>
       <c r="V24" s="0"/>
       <c r="W24" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C24="","Missing blog title",""),IF(E24="","Missing slides per post",""),IF(OR(E24&lt;1,E24&gt;10),"Slides per post must be 1-10",""),IF(F24="","Missing URL",""),IF(G24="","Missing width",""),IF(H24="","Missing height",""),IF(I24="","Missing theme",""),IF(M24="","Missing hero type",""),IF(N24="","Missing image direction",""),IF(U24="","Missing status",""),IF(AND(J24="Custom",K24=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C24="","Missing blog title",""),IF(E24="","Missing URL",""),IF(F24="","Missing number of slides",""),IF(OR(F24&lt;1,F24&gt;10),"Number of slides must be 1-10",""),IF(G24="","Missing width",""),IF(H24="","Missing height",""),IF(I24="","Missing theme",""),IF(M24="","Missing hero type",""),IF(N24="","Missing image direction",""),IF(U24="","Missing status",""),IF(AND(J24="Custom",K24=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="25">
@@ -1669,10 +1652,10 @@
       <c r="B25" s="0"/>
       <c r="C25" s="0"/>
       <c r="D25" s="0"/>
-      <c r="E25" s="0">
-        <v>1</v>
-      </c>
-      <c r="F25" s="0"/>
+      <c r="E25" s="0"/>
+      <c r="F25" s="0">
+        <v>1</v>
+      </c>
       <c r="G25" s="0">
         <v>1000</v>
       </c>
@@ -1714,7 +1697,7 @@
       </c>
       <c r="V25" s="0"/>
       <c r="W25" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C25="","Missing blog title",""),IF(E25="","Missing slides per post",""),IF(OR(E25&lt;1,E25&gt;10),"Slides per post must be 1-10",""),IF(F25="","Missing URL",""),IF(G25="","Missing width",""),IF(H25="","Missing height",""),IF(I25="","Missing theme",""),IF(M25="","Missing hero type",""),IF(N25="","Missing image direction",""),IF(U25="","Missing status",""),IF(AND(J25="Custom",K25=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C25="","Missing blog title",""),IF(E25="","Missing URL",""),IF(F25="","Missing number of slides",""),IF(OR(F25&lt;1,F25&gt;10),"Number of slides must be 1-10",""),IF(G25="","Missing width",""),IF(H25="","Missing height",""),IF(I25="","Missing theme",""),IF(M25="","Missing hero type",""),IF(N25="","Missing image direction",""),IF(U25="","Missing status",""),IF(AND(J25="Custom",K25=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="26">
@@ -1724,10 +1707,10 @@
       <c r="B26" s="0"/>
       <c r="C26" s="0"/>
       <c r="D26" s="0"/>
-      <c r="E26" s="0">
-        <v>1</v>
-      </c>
-      <c r="F26" s="0"/>
+      <c r="E26" s="0"/>
+      <c r="F26" s="0">
+        <v>1</v>
+      </c>
       <c r="G26" s="0">
         <v>1000</v>
       </c>
@@ -1769,7 +1752,7 @@
       </c>
       <c r="V26" s="0"/>
       <c r="W26" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C26="","Missing blog title",""),IF(E26="","Missing slides per post",""),IF(OR(E26&lt;1,E26&gt;10),"Slides per post must be 1-10",""),IF(F26="","Missing URL",""),IF(G26="","Missing width",""),IF(H26="","Missing height",""),IF(I26="","Missing theme",""),IF(M26="","Missing hero type",""),IF(N26="","Missing image direction",""),IF(U26="","Missing status",""),IF(AND(J26="Custom",K26=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C26="","Missing blog title",""),IF(E26="","Missing URL",""),IF(F26="","Missing number of slides",""),IF(OR(F26&lt;1,F26&gt;10),"Number of slides must be 1-10",""),IF(G26="","Missing width",""),IF(H26="","Missing height",""),IF(I26="","Missing theme",""),IF(M26="","Missing hero type",""),IF(N26="","Missing image direction",""),IF(U26="","Missing status",""),IF(AND(J26="Custom",K26=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="27">
@@ -1779,10 +1762,10 @@
       <c r="B27" s="0"/>
       <c r="C27" s="0"/>
       <c r="D27" s="0"/>
-      <c r="E27" s="0">
-        <v>1</v>
-      </c>
-      <c r="F27" s="0"/>
+      <c r="E27" s="0"/>
+      <c r="F27" s="0">
+        <v>1</v>
+      </c>
       <c r="G27" s="0">
         <v>1000</v>
       </c>
@@ -1824,7 +1807,7 @@
       </c>
       <c r="V27" s="0"/>
       <c r="W27" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C27="","Missing blog title",""),IF(E27="","Missing slides per post",""),IF(OR(E27&lt;1,E27&gt;10),"Slides per post must be 1-10",""),IF(F27="","Missing URL",""),IF(G27="","Missing width",""),IF(H27="","Missing height",""),IF(I27="","Missing theme",""),IF(M27="","Missing hero type",""),IF(N27="","Missing image direction",""),IF(U27="","Missing status",""),IF(AND(J27="Custom",K27=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C27="","Missing blog title",""),IF(E27="","Missing URL",""),IF(F27="","Missing number of slides",""),IF(OR(F27&lt;1,F27&gt;10),"Number of slides must be 1-10",""),IF(G27="","Missing width",""),IF(H27="","Missing height",""),IF(I27="","Missing theme",""),IF(M27="","Missing hero type",""),IF(N27="","Missing image direction",""),IF(U27="","Missing status",""),IF(AND(J27="Custom",K27=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="28">
@@ -1834,10 +1817,10 @@
       <c r="B28" s="0"/>
       <c r="C28" s="0"/>
       <c r="D28" s="0"/>
-      <c r="E28" s="0">
-        <v>1</v>
-      </c>
-      <c r="F28" s="0"/>
+      <c r="E28" s="0"/>
+      <c r="F28" s="0">
+        <v>1</v>
+      </c>
       <c r="G28" s="0">
         <v>1000</v>
       </c>
@@ -1879,7 +1862,7 @@
       </c>
       <c r="V28" s="0"/>
       <c r="W28" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C28="","Missing blog title",""),IF(E28="","Missing slides per post",""),IF(OR(E28&lt;1,E28&gt;10),"Slides per post must be 1-10",""),IF(F28="","Missing URL",""),IF(G28="","Missing width",""),IF(H28="","Missing height",""),IF(I28="","Missing theme",""),IF(M28="","Missing hero type",""),IF(N28="","Missing image direction",""),IF(U28="","Missing status",""),IF(AND(J28="Custom",K28=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C28="","Missing blog title",""),IF(E28="","Missing URL",""),IF(F28="","Missing number of slides",""),IF(OR(F28&lt;1,F28&gt;10),"Number of slides must be 1-10",""),IF(G28="","Missing width",""),IF(H28="","Missing height",""),IF(I28="","Missing theme",""),IF(M28="","Missing hero type",""),IF(N28="","Missing image direction",""),IF(U28="","Missing status",""),IF(AND(J28="Custom",K28=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="29">
@@ -1889,10 +1872,10 @@
       <c r="B29" s="0"/>
       <c r="C29" s="0"/>
       <c r="D29" s="0"/>
-      <c r="E29" s="0">
-        <v>1</v>
-      </c>
-      <c r="F29" s="0"/>
+      <c r="E29" s="0"/>
+      <c r="F29" s="0">
+        <v>1</v>
+      </c>
       <c r="G29" s="0">
         <v>1000</v>
       </c>
@@ -1934,7 +1917,7 @@
       </c>
       <c r="V29" s="0"/>
       <c r="W29" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C29="","Missing blog title",""),IF(E29="","Missing slides per post",""),IF(OR(E29&lt;1,E29&gt;10),"Slides per post must be 1-10",""),IF(F29="","Missing URL",""),IF(G29="","Missing width",""),IF(H29="","Missing height",""),IF(I29="","Missing theme",""),IF(M29="","Missing hero type",""),IF(N29="","Missing image direction",""),IF(U29="","Missing status",""),IF(AND(J29="Custom",K29=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C29="","Missing blog title",""),IF(E29="","Missing URL",""),IF(F29="","Missing number of slides",""),IF(OR(F29&lt;1,F29&gt;10),"Number of slides must be 1-10",""),IF(G29="","Missing width",""),IF(H29="","Missing height",""),IF(I29="","Missing theme",""),IF(M29="","Missing hero type",""),IF(N29="","Missing image direction",""),IF(U29="","Missing status",""),IF(AND(J29="Custom",K29=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="30">
@@ -1944,10 +1927,10 @@
       <c r="B30" s="0"/>
       <c r="C30" s="0"/>
       <c r="D30" s="0"/>
-      <c r="E30" s="0">
-        <v>1</v>
-      </c>
-      <c r="F30" s="0"/>
+      <c r="E30" s="0"/>
+      <c r="F30" s="0">
+        <v>1</v>
+      </c>
       <c r="G30" s="0">
         <v>1000</v>
       </c>
@@ -1989,7 +1972,7 @@
       </c>
       <c r="V30" s="0"/>
       <c r="W30" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C30="","Missing blog title",""),IF(E30="","Missing slides per post",""),IF(OR(E30&lt;1,E30&gt;10),"Slides per post must be 1-10",""),IF(F30="","Missing URL",""),IF(G30="","Missing width",""),IF(H30="","Missing height",""),IF(I30="","Missing theme",""),IF(M30="","Missing hero type",""),IF(N30="","Missing image direction",""),IF(U30="","Missing status",""),IF(AND(J30="Custom",K30=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C30="","Missing blog title",""),IF(E30="","Missing URL",""),IF(F30="","Missing number of slides",""),IF(OR(F30&lt;1,F30&gt;10),"Number of slides must be 1-10",""),IF(G30="","Missing width",""),IF(H30="","Missing height",""),IF(I30="","Missing theme",""),IF(M30="","Missing hero type",""),IF(N30="","Missing image direction",""),IF(U30="","Missing status",""),IF(AND(J30="Custom",K30=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="31">
@@ -1999,10 +1982,10 @@
       <c r="B31" s="0"/>
       <c r="C31" s="0"/>
       <c r="D31" s="0"/>
-      <c r="E31" s="0">
-        <v>1</v>
-      </c>
-      <c r="F31" s="0"/>
+      <c r="E31" s="0"/>
+      <c r="F31" s="0">
+        <v>1</v>
+      </c>
       <c r="G31" s="0">
         <v>1000</v>
       </c>
@@ -2044,7 +2027,7 @@
       </c>
       <c r="V31" s="0"/>
       <c r="W31" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C31="","Missing blog title",""),IF(E31="","Missing slides per post",""),IF(OR(E31&lt;1,E31&gt;10),"Slides per post must be 1-10",""),IF(F31="","Missing URL",""),IF(G31="","Missing width",""),IF(H31="","Missing height",""),IF(I31="","Missing theme",""),IF(M31="","Missing hero type",""),IF(N31="","Missing image direction",""),IF(U31="","Missing status",""),IF(AND(J31="Custom",K31=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C31="","Missing blog title",""),IF(E31="","Missing URL",""),IF(F31="","Missing number of slides",""),IF(OR(F31&lt;1,F31&gt;10),"Number of slides must be 1-10",""),IF(G31="","Missing width",""),IF(H31="","Missing height",""),IF(I31="","Missing theme",""),IF(M31="","Missing hero type",""),IF(N31="","Missing image direction",""),IF(U31="","Missing status",""),IF(AND(J31="Custom",K31=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="32">
@@ -2054,10 +2037,10 @@
       <c r="B32" s="0"/>
       <c r="C32" s="0"/>
       <c r="D32" s="0"/>
-      <c r="E32" s="0">
-        <v>1</v>
-      </c>
-      <c r="F32" s="0"/>
+      <c r="E32" s="0"/>
+      <c r="F32" s="0">
+        <v>1</v>
+      </c>
       <c r="G32" s="0">
         <v>1000</v>
       </c>
@@ -2099,7 +2082,7 @@
       </c>
       <c r="V32" s="0"/>
       <c r="W32" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C32="","Missing blog title",""),IF(E32="","Missing slides per post",""),IF(OR(E32&lt;1,E32&gt;10),"Slides per post must be 1-10",""),IF(F32="","Missing URL",""),IF(G32="","Missing width",""),IF(H32="","Missing height",""),IF(I32="","Missing theme",""),IF(M32="","Missing hero type",""),IF(N32="","Missing image direction",""),IF(U32="","Missing status",""),IF(AND(J32="Custom",K32=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C32="","Missing blog title",""),IF(E32="","Missing URL",""),IF(F32="","Missing number of slides",""),IF(OR(F32&lt;1,F32&gt;10),"Number of slides must be 1-10",""),IF(G32="","Missing width",""),IF(H32="","Missing height",""),IF(I32="","Missing theme",""),IF(M32="","Missing hero type",""),IF(N32="","Missing image direction",""),IF(U32="","Missing status",""),IF(AND(J32="Custom",K32=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="33">
@@ -2109,10 +2092,10 @@
       <c r="B33" s="0"/>
       <c r="C33" s="0"/>
       <c r="D33" s="0"/>
-      <c r="E33" s="0">
-        <v>1</v>
-      </c>
-      <c r="F33" s="0"/>
+      <c r="E33" s="0"/>
+      <c r="F33" s="0">
+        <v>1</v>
+      </c>
       <c r="G33" s="0">
         <v>1000</v>
       </c>
@@ -2154,7 +2137,7 @@
       </c>
       <c r="V33" s="0"/>
       <c r="W33" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C33="","Missing blog title",""),IF(E33="","Missing slides per post",""),IF(OR(E33&lt;1,E33&gt;10),"Slides per post must be 1-10",""),IF(F33="","Missing URL",""),IF(G33="","Missing width",""),IF(H33="","Missing height",""),IF(I33="","Missing theme",""),IF(M33="","Missing hero type",""),IF(N33="","Missing image direction",""),IF(U33="","Missing status",""),IF(AND(J33="Custom",K33=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C33="","Missing blog title",""),IF(E33="","Missing URL",""),IF(F33="","Missing number of slides",""),IF(OR(F33&lt;1,F33&gt;10),"Number of slides must be 1-10",""),IF(G33="","Missing width",""),IF(H33="","Missing height",""),IF(I33="","Missing theme",""),IF(M33="","Missing hero type",""),IF(N33="","Missing image direction",""),IF(U33="","Missing status",""),IF(AND(J33="Custom",K33=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="34">
@@ -2164,10 +2147,10 @@
       <c r="B34" s="0"/>
       <c r="C34" s="0"/>
       <c r="D34" s="0"/>
-      <c r="E34" s="0">
-        <v>1</v>
-      </c>
-      <c r="F34" s="0"/>
+      <c r="E34" s="0"/>
+      <c r="F34" s="0">
+        <v>1</v>
+      </c>
       <c r="G34" s="0">
         <v>1000</v>
       </c>
@@ -2209,7 +2192,7 @@
       </c>
       <c r="V34" s="0"/>
       <c r="W34" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C34="","Missing blog title",""),IF(E34="","Missing slides per post",""),IF(OR(E34&lt;1,E34&gt;10),"Slides per post must be 1-10",""),IF(F34="","Missing URL",""),IF(G34="","Missing width",""),IF(H34="","Missing height",""),IF(I34="","Missing theme",""),IF(M34="","Missing hero type",""),IF(N34="","Missing image direction",""),IF(U34="","Missing status",""),IF(AND(J34="Custom",K34=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C34="","Missing blog title",""),IF(E34="","Missing URL",""),IF(F34="","Missing number of slides",""),IF(OR(F34&lt;1,F34&gt;10),"Number of slides must be 1-10",""),IF(G34="","Missing width",""),IF(H34="","Missing height",""),IF(I34="","Missing theme",""),IF(M34="","Missing hero type",""),IF(N34="","Missing image direction",""),IF(U34="","Missing status",""),IF(AND(J34="Custom",K34=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="35">
@@ -2219,10 +2202,10 @@
       <c r="B35" s="0"/>
       <c r="C35" s="0"/>
       <c r="D35" s="0"/>
-      <c r="E35" s="0">
-        <v>1</v>
-      </c>
-      <c r="F35" s="0"/>
+      <c r="E35" s="0"/>
+      <c r="F35" s="0">
+        <v>1</v>
+      </c>
       <c r="G35" s="0">
         <v>1000</v>
       </c>
@@ -2264,7 +2247,7 @@
       </c>
       <c r="V35" s="0"/>
       <c r="W35" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C35="","Missing blog title",""),IF(E35="","Missing slides per post",""),IF(OR(E35&lt;1,E35&gt;10),"Slides per post must be 1-10",""),IF(F35="","Missing URL",""),IF(G35="","Missing width",""),IF(H35="","Missing height",""),IF(I35="","Missing theme",""),IF(M35="","Missing hero type",""),IF(N35="","Missing image direction",""),IF(U35="","Missing status",""),IF(AND(J35="Custom",K35=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C35="","Missing blog title",""),IF(E35="","Missing URL",""),IF(F35="","Missing number of slides",""),IF(OR(F35&lt;1,F35&gt;10),"Number of slides must be 1-10",""),IF(G35="","Missing width",""),IF(H35="","Missing height",""),IF(I35="","Missing theme",""),IF(M35="","Missing hero type",""),IF(N35="","Missing image direction",""),IF(U35="","Missing status",""),IF(AND(J35="Custom",K35=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="36">
@@ -2274,10 +2257,10 @@
       <c r="B36" s="0"/>
       <c r="C36" s="0"/>
       <c r="D36" s="0"/>
-      <c r="E36" s="0">
-        <v>1</v>
-      </c>
-      <c r="F36" s="0"/>
+      <c r="E36" s="0"/>
+      <c r="F36" s="0">
+        <v>1</v>
+      </c>
       <c r="G36" s="0">
         <v>1000</v>
       </c>
@@ -2319,7 +2302,7 @@
       </c>
       <c r="V36" s="0"/>
       <c r="W36" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C36="","Missing blog title",""),IF(E36="","Missing slides per post",""),IF(OR(E36&lt;1,E36&gt;10),"Slides per post must be 1-10",""),IF(F36="","Missing URL",""),IF(G36="","Missing width",""),IF(H36="","Missing height",""),IF(I36="","Missing theme",""),IF(M36="","Missing hero type",""),IF(N36="","Missing image direction",""),IF(U36="","Missing status",""),IF(AND(J36="Custom",K36=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C36="","Missing blog title",""),IF(E36="","Missing URL",""),IF(F36="","Missing number of slides",""),IF(OR(F36&lt;1,F36&gt;10),"Number of slides must be 1-10",""),IF(G36="","Missing width",""),IF(H36="","Missing height",""),IF(I36="","Missing theme",""),IF(M36="","Missing hero type",""),IF(N36="","Missing image direction",""),IF(U36="","Missing status",""),IF(AND(J36="Custom",K36=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="37">
@@ -2329,10 +2312,10 @@
       <c r="B37" s="0"/>
       <c r="C37" s="0"/>
       <c r="D37" s="0"/>
-      <c r="E37" s="0">
-        <v>1</v>
-      </c>
-      <c r="F37" s="0"/>
+      <c r="E37" s="0"/>
+      <c r="F37" s="0">
+        <v>1</v>
+      </c>
       <c r="G37" s="0">
         <v>1000</v>
       </c>
@@ -2374,7 +2357,7 @@
       </c>
       <c r="V37" s="0"/>
       <c r="W37" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C37="","Missing blog title",""),IF(E37="","Missing slides per post",""),IF(OR(E37&lt;1,E37&gt;10),"Slides per post must be 1-10",""),IF(F37="","Missing URL",""),IF(G37="","Missing width",""),IF(H37="","Missing height",""),IF(I37="","Missing theme",""),IF(M37="","Missing hero type",""),IF(N37="","Missing image direction",""),IF(U37="","Missing status",""),IF(AND(J37="Custom",K37=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C37="","Missing blog title",""),IF(E37="","Missing URL",""),IF(F37="","Missing number of slides",""),IF(OR(F37&lt;1,F37&gt;10),"Number of slides must be 1-10",""),IF(G37="","Missing width",""),IF(H37="","Missing height",""),IF(I37="","Missing theme",""),IF(M37="","Missing hero type",""),IF(N37="","Missing image direction",""),IF(U37="","Missing status",""),IF(AND(J37="Custom",K37=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="38">
@@ -2384,10 +2367,10 @@
       <c r="B38" s="0"/>
       <c r="C38" s="0"/>
       <c r="D38" s="0"/>
-      <c r="E38" s="0">
-        <v>1</v>
-      </c>
-      <c r="F38" s="0"/>
+      <c r="E38" s="0"/>
+      <c r="F38" s="0">
+        <v>1</v>
+      </c>
       <c r="G38" s="0">
         <v>1000</v>
       </c>
@@ -2429,7 +2412,7 @@
       </c>
       <c r="V38" s="0"/>
       <c r="W38" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C38="","Missing blog title",""),IF(E38="","Missing slides per post",""),IF(OR(E38&lt;1,E38&gt;10),"Slides per post must be 1-10",""),IF(F38="","Missing URL",""),IF(G38="","Missing width",""),IF(H38="","Missing height",""),IF(I38="","Missing theme",""),IF(M38="","Missing hero type",""),IF(N38="","Missing image direction",""),IF(U38="","Missing status",""),IF(AND(J38="Custom",K38=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C38="","Missing blog title",""),IF(E38="","Missing URL",""),IF(F38="","Missing number of slides",""),IF(OR(F38&lt;1,F38&gt;10),"Number of slides must be 1-10",""),IF(G38="","Missing width",""),IF(H38="","Missing height",""),IF(I38="","Missing theme",""),IF(M38="","Missing hero type",""),IF(N38="","Missing image direction",""),IF(U38="","Missing status",""),IF(AND(J38="Custom",K38=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="39">
@@ -2439,10 +2422,10 @@
       <c r="B39" s="0"/>
       <c r="C39" s="0"/>
       <c r="D39" s="0"/>
-      <c r="E39" s="0">
-        <v>1</v>
-      </c>
-      <c r="F39" s="0"/>
+      <c r="E39" s="0"/>
+      <c r="F39" s="0">
+        <v>1</v>
+      </c>
       <c r="G39" s="0">
         <v>1000</v>
       </c>
@@ -2484,7 +2467,7 @@
       </c>
       <c r="V39" s="0"/>
       <c r="W39" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C39="","Missing blog title",""),IF(E39="","Missing slides per post",""),IF(OR(E39&lt;1,E39&gt;10),"Slides per post must be 1-10",""),IF(F39="","Missing URL",""),IF(G39="","Missing width",""),IF(H39="","Missing height",""),IF(I39="","Missing theme",""),IF(M39="","Missing hero type",""),IF(N39="","Missing image direction",""),IF(U39="","Missing status",""),IF(AND(J39="Custom",K39=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C39="","Missing blog title",""),IF(E39="","Missing URL",""),IF(F39="","Missing number of slides",""),IF(OR(F39&lt;1,F39&gt;10),"Number of slides must be 1-10",""),IF(G39="","Missing width",""),IF(H39="","Missing height",""),IF(I39="","Missing theme",""),IF(M39="","Missing hero type",""),IF(N39="","Missing image direction",""),IF(U39="","Missing status",""),IF(AND(J39="Custom",K39=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="40">
@@ -2494,10 +2477,10 @@
       <c r="B40" s="0"/>
       <c r="C40" s="0"/>
       <c r="D40" s="0"/>
-      <c r="E40" s="0">
-        <v>1</v>
-      </c>
-      <c r="F40" s="0"/>
+      <c r="E40" s="0"/>
+      <c r="F40" s="0">
+        <v>1</v>
+      </c>
       <c r="G40" s="0">
         <v>1000</v>
       </c>
@@ -2539,7 +2522,7 @@
       </c>
       <c r="V40" s="0"/>
       <c r="W40" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C40="","Missing blog title",""),IF(E40="","Missing slides per post",""),IF(OR(E40&lt;1,E40&gt;10),"Slides per post must be 1-10",""),IF(F40="","Missing URL",""),IF(G40="","Missing width",""),IF(H40="","Missing height",""),IF(I40="","Missing theme",""),IF(M40="","Missing hero type",""),IF(N40="","Missing image direction",""),IF(U40="","Missing status",""),IF(AND(J40="Custom",K40=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C40="","Missing blog title",""),IF(E40="","Missing URL",""),IF(F40="","Missing number of slides",""),IF(OR(F40&lt;1,F40&gt;10),"Number of slides must be 1-10",""),IF(G40="","Missing width",""),IF(H40="","Missing height",""),IF(I40="","Missing theme",""),IF(M40="","Missing hero type",""),IF(N40="","Missing image direction",""),IF(U40="","Missing status",""),IF(AND(J40="Custom",K40=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="41">
@@ -2549,10 +2532,10 @@
       <c r="B41" s="0"/>
       <c r="C41" s="0"/>
       <c r="D41" s="0"/>
-      <c r="E41" s="0">
-        <v>1</v>
-      </c>
-      <c r="F41" s="0"/>
+      <c r="E41" s="0"/>
+      <c r="F41" s="0">
+        <v>1</v>
+      </c>
       <c r="G41" s="0">
         <v>1000</v>
       </c>
@@ -2594,7 +2577,7 @@
       </c>
       <c r="V41" s="0"/>
       <c r="W41" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C41="","Missing blog title",""),IF(E41="","Missing slides per post",""),IF(OR(E41&lt;1,E41&gt;10),"Slides per post must be 1-10",""),IF(F41="","Missing URL",""),IF(G41="","Missing width",""),IF(H41="","Missing height",""),IF(I41="","Missing theme",""),IF(M41="","Missing hero type",""),IF(N41="","Missing image direction",""),IF(U41="","Missing status",""),IF(AND(J41="Custom",K41=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C41="","Missing blog title",""),IF(E41="","Missing URL",""),IF(F41="","Missing number of slides",""),IF(OR(F41&lt;1,F41&gt;10),"Number of slides must be 1-10",""),IF(G41="","Missing width",""),IF(H41="","Missing height",""),IF(I41="","Missing theme",""),IF(M41="","Missing hero type",""),IF(N41="","Missing image direction",""),IF(U41="","Missing status",""),IF(AND(J41="Custom",K41=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="42">
@@ -2604,10 +2587,10 @@
       <c r="B42" s="0"/>
       <c r="C42" s="0"/>
       <c r="D42" s="0"/>
-      <c r="E42" s="0">
-        <v>1</v>
-      </c>
-      <c r="F42" s="0"/>
+      <c r="E42" s="0"/>
+      <c r="F42" s="0">
+        <v>1</v>
+      </c>
       <c r="G42" s="0">
         <v>1000</v>
       </c>
@@ -2649,7 +2632,7 @@
       </c>
       <c r="V42" s="0"/>
       <c r="W42" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C42="","Missing blog title",""),IF(E42="","Missing slides per post",""),IF(OR(E42&lt;1,E42&gt;10),"Slides per post must be 1-10",""),IF(F42="","Missing URL",""),IF(G42="","Missing width",""),IF(H42="","Missing height",""),IF(I42="","Missing theme",""),IF(M42="","Missing hero type",""),IF(N42="","Missing image direction",""),IF(U42="","Missing status",""),IF(AND(J42="Custom",K42=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C42="","Missing blog title",""),IF(E42="","Missing URL",""),IF(F42="","Missing number of slides",""),IF(OR(F42&lt;1,F42&gt;10),"Number of slides must be 1-10",""),IF(G42="","Missing width",""),IF(H42="","Missing height",""),IF(I42="","Missing theme",""),IF(M42="","Missing hero type",""),IF(N42="","Missing image direction",""),IF(U42="","Missing status",""),IF(AND(J42="Custom",K42=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="43">
@@ -2659,10 +2642,10 @@
       <c r="B43" s="0"/>
       <c r="C43" s="0"/>
       <c r="D43" s="0"/>
-      <c r="E43" s="0">
-        <v>1</v>
-      </c>
-      <c r="F43" s="0"/>
+      <c r="E43" s="0"/>
+      <c r="F43" s="0">
+        <v>1</v>
+      </c>
       <c r="G43" s="0">
         <v>1000</v>
       </c>
@@ -2704,7 +2687,7 @@
       </c>
       <c r="V43" s="0"/>
       <c r="W43" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C43="","Missing blog title",""),IF(E43="","Missing slides per post",""),IF(OR(E43&lt;1,E43&gt;10),"Slides per post must be 1-10",""),IF(F43="","Missing URL",""),IF(G43="","Missing width",""),IF(H43="","Missing height",""),IF(I43="","Missing theme",""),IF(M43="","Missing hero type",""),IF(N43="","Missing image direction",""),IF(U43="","Missing status",""),IF(AND(J43="Custom",K43=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C43="","Missing blog title",""),IF(E43="","Missing URL",""),IF(F43="","Missing number of slides",""),IF(OR(F43&lt;1,F43&gt;10),"Number of slides must be 1-10",""),IF(G43="","Missing width",""),IF(H43="","Missing height",""),IF(I43="","Missing theme",""),IF(M43="","Missing hero type",""),IF(N43="","Missing image direction",""),IF(U43="","Missing status",""),IF(AND(J43="Custom",K43=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="44">
@@ -2714,10 +2697,10 @@
       <c r="B44" s="0"/>
       <c r="C44" s="0"/>
       <c r="D44" s="0"/>
-      <c r="E44" s="0">
-        <v>1</v>
-      </c>
-      <c r="F44" s="0"/>
+      <c r="E44" s="0"/>
+      <c r="F44" s="0">
+        <v>1</v>
+      </c>
       <c r="G44" s="0">
         <v>1000</v>
       </c>
@@ -2759,7 +2742,7 @@
       </c>
       <c r="V44" s="0"/>
       <c r="W44" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C44="","Missing blog title",""),IF(E44="","Missing slides per post",""),IF(OR(E44&lt;1,E44&gt;10),"Slides per post must be 1-10",""),IF(F44="","Missing URL",""),IF(G44="","Missing width",""),IF(H44="","Missing height",""),IF(I44="","Missing theme",""),IF(M44="","Missing hero type",""),IF(N44="","Missing image direction",""),IF(U44="","Missing status",""),IF(AND(J44="Custom",K44=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C44="","Missing blog title",""),IF(E44="","Missing URL",""),IF(F44="","Missing number of slides",""),IF(OR(F44&lt;1,F44&gt;10),"Number of slides must be 1-10",""),IF(G44="","Missing width",""),IF(H44="","Missing height",""),IF(I44="","Missing theme",""),IF(M44="","Missing hero type",""),IF(N44="","Missing image direction",""),IF(U44="","Missing status",""),IF(AND(J44="Custom",K44=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="45">
@@ -2769,10 +2752,10 @@
       <c r="B45" s="0"/>
       <c r="C45" s="0"/>
       <c r="D45" s="0"/>
-      <c r="E45" s="0">
-        <v>1</v>
-      </c>
-      <c r="F45" s="0"/>
+      <c r="E45" s="0"/>
+      <c r="F45" s="0">
+        <v>1</v>
+      </c>
       <c r="G45" s="0">
         <v>1000</v>
       </c>
@@ -2814,7 +2797,7 @@
       </c>
       <c r="V45" s="0"/>
       <c r="W45" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C45="","Missing blog title",""),IF(E45="","Missing slides per post",""),IF(OR(E45&lt;1,E45&gt;10),"Slides per post must be 1-10",""),IF(F45="","Missing URL",""),IF(G45="","Missing width",""),IF(H45="","Missing height",""),IF(I45="","Missing theme",""),IF(M45="","Missing hero type",""),IF(N45="","Missing image direction",""),IF(U45="","Missing status",""),IF(AND(J45="Custom",K45=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C45="","Missing blog title",""),IF(E45="","Missing URL",""),IF(F45="","Missing number of slides",""),IF(OR(F45&lt;1,F45&gt;10),"Number of slides must be 1-10",""),IF(G45="","Missing width",""),IF(H45="","Missing height",""),IF(I45="","Missing theme",""),IF(M45="","Missing hero type",""),IF(N45="","Missing image direction",""),IF(U45="","Missing status",""),IF(AND(J45="Custom",K45=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="46">
@@ -2824,10 +2807,10 @@
       <c r="B46" s="0"/>
       <c r="C46" s="0"/>
       <c r="D46" s="0"/>
-      <c r="E46" s="0">
-        <v>1</v>
-      </c>
-      <c r="F46" s="0"/>
+      <c r="E46" s="0"/>
+      <c r="F46" s="0">
+        <v>1</v>
+      </c>
       <c r="G46" s="0">
         <v>1000</v>
       </c>
@@ -2869,7 +2852,7 @@
       </c>
       <c r="V46" s="0"/>
       <c r="W46" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C46="","Missing blog title",""),IF(E46="","Missing slides per post",""),IF(OR(E46&lt;1,E46&gt;10),"Slides per post must be 1-10",""),IF(F46="","Missing URL",""),IF(G46="","Missing width",""),IF(H46="","Missing height",""),IF(I46="","Missing theme",""),IF(M46="","Missing hero type",""),IF(N46="","Missing image direction",""),IF(U46="","Missing status",""),IF(AND(J46="Custom",K46=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C46="","Missing blog title",""),IF(E46="","Missing URL",""),IF(F46="","Missing number of slides",""),IF(OR(F46&lt;1,F46&gt;10),"Number of slides must be 1-10",""),IF(G46="","Missing width",""),IF(H46="","Missing height",""),IF(I46="","Missing theme",""),IF(M46="","Missing hero type",""),IF(N46="","Missing image direction",""),IF(U46="","Missing status",""),IF(AND(J46="Custom",K46=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="47">
@@ -2879,10 +2862,10 @@
       <c r="B47" s="0"/>
       <c r="C47" s="0"/>
       <c r="D47" s="0"/>
-      <c r="E47" s="0">
-        <v>1</v>
-      </c>
-      <c r="F47" s="0"/>
+      <c r="E47" s="0"/>
+      <c r="F47" s="0">
+        <v>1</v>
+      </c>
       <c r="G47" s="0">
         <v>1000</v>
       </c>
@@ -2924,7 +2907,7 @@
       </c>
       <c r="V47" s="0"/>
       <c r="W47" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C47="","Missing blog title",""),IF(E47="","Missing slides per post",""),IF(OR(E47&lt;1,E47&gt;10),"Slides per post must be 1-10",""),IF(F47="","Missing URL",""),IF(G47="","Missing width",""),IF(H47="","Missing height",""),IF(I47="","Missing theme",""),IF(M47="","Missing hero type",""),IF(N47="","Missing image direction",""),IF(U47="","Missing status",""),IF(AND(J47="Custom",K47=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C47="","Missing blog title",""),IF(E47="","Missing URL",""),IF(F47="","Missing number of slides",""),IF(OR(F47&lt;1,F47&gt;10),"Number of slides must be 1-10",""),IF(G47="","Missing width",""),IF(H47="","Missing height",""),IF(I47="","Missing theme",""),IF(M47="","Missing hero type",""),IF(N47="","Missing image direction",""),IF(U47="","Missing status",""),IF(AND(J47="Custom",K47=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="48">
@@ -2934,10 +2917,10 @@
       <c r="B48" s="0"/>
       <c r="C48" s="0"/>
       <c r="D48" s="0"/>
-      <c r="E48" s="0">
-        <v>1</v>
-      </c>
-      <c r="F48" s="0"/>
+      <c r="E48" s="0"/>
+      <c r="F48" s="0">
+        <v>1</v>
+      </c>
       <c r="G48" s="0">
         <v>1000</v>
       </c>
@@ -2979,7 +2962,7 @@
       </c>
       <c r="V48" s="0"/>
       <c r="W48" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C48="","Missing blog title",""),IF(E48="","Missing slides per post",""),IF(OR(E48&lt;1,E48&gt;10),"Slides per post must be 1-10",""),IF(F48="","Missing URL",""),IF(G48="","Missing width",""),IF(H48="","Missing height",""),IF(I48="","Missing theme",""),IF(M48="","Missing hero type",""),IF(N48="","Missing image direction",""),IF(U48="","Missing status",""),IF(AND(J48="Custom",K48=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C48="","Missing blog title",""),IF(E48="","Missing URL",""),IF(F48="","Missing number of slides",""),IF(OR(F48&lt;1,F48&gt;10),"Number of slides must be 1-10",""),IF(G48="","Missing width",""),IF(H48="","Missing height",""),IF(I48="","Missing theme",""),IF(M48="","Missing hero type",""),IF(N48="","Missing image direction",""),IF(U48="","Missing status",""),IF(AND(J48="Custom",K48=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="49">
@@ -2989,10 +2972,10 @@
       <c r="B49" s="0"/>
       <c r="C49" s="0"/>
       <c r="D49" s="0"/>
-      <c r="E49" s="0">
-        <v>1</v>
-      </c>
-      <c r="F49" s="0"/>
+      <c r="E49" s="0"/>
+      <c r="F49" s="0">
+        <v>1</v>
+      </c>
       <c r="G49" s="0">
         <v>1000</v>
       </c>
@@ -3034,7 +3017,7 @@
       </c>
       <c r="V49" s="0"/>
       <c r="W49" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C49="","Missing blog title",""),IF(E49="","Missing slides per post",""),IF(OR(E49&lt;1,E49&gt;10),"Slides per post must be 1-10",""),IF(F49="","Missing URL",""),IF(G49="","Missing width",""),IF(H49="","Missing height",""),IF(I49="","Missing theme",""),IF(M49="","Missing hero type",""),IF(N49="","Missing image direction",""),IF(U49="","Missing status",""),IF(AND(J49="Custom",K49=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C49="","Missing blog title",""),IF(E49="","Missing URL",""),IF(F49="","Missing number of slides",""),IF(OR(F49&lt;1,F49&gt;10),"Number of slides must be 1-10",""),IF(G49="","Missing width",""),IF(H49="","Missing height",""),IF(I49="","Missing theme",""),IF(M49="","Missing hero type",""),IF(N49="","Missing image direction",""),IF(U49="","Missing status",""),IF(AND(J49="Custom",K49=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="50">
@@ -3044,10 +3027,10 @@
       <c r="B50" s="0"/>
       <c r="C50" s="0"/>
       <c r="D50" s="0"/>
-      <c r="E50" s="0">
-        <v>1</v>
-      </c>
-      <c r="F50" s="0"/>
+      <c r="E50" s="0"/>
+      <c r="F50" s="0">
+        <v>1</v>
+      </c>
       <c r="G50" s="0">
         <v>1000</v>
       </c>
@@ -3089,7 +3072,7 @@
       </c>
       <c r="V50" s="0"/>
       <c r="W50" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C50="","Missing blog title",""),IF(E50="","Missing slides per post",""),IF(OR(E50&lt;1,E50&gt;10),"Slides per post must be 1-10",""),IF(F50="","Missing URL",""),IF(G50="","Missing width",""),IF(H50="","Missing height",""),IF(I50="","Missing theme",""),IF(M50="","Missing hero type",""),IF(N50="","Missing image direction",""),IF(U50="","Missing status",""),IF(AND(J50="Custom",K50=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C50="","Missing blog title",""),IF(E50="","Missing URL",""),IF(F50="","Missing number of slides",""),IF(OR(F50&lt;1,F50&gt;10),"Number of slides must be 1-10",""),IF(G50="","Missing width",""),IF(H50="","Missing height",""),IF(I50="","Missing theme",""),IF(M50="","Missing hero type",""),IF(N50="","Missing image direction",""),IF(U50="","Missing status",""),IF(AND(J50="Custom",K50=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="51">
@@ -3099,10 +3082,10 @@
       <c r="B51" s="0"/>
       <c r="C51" s="0"/>
       <c r="D51" s="0"/>
-      <c r="E51" s="0">
-        <v>1</v>
-      </c>
-      <c r="F51" s="0"/>
+      <c r="E51" s="0"/>
+      <c r="F51" s="0">
+        <v>1</v>
+      </c>
       <c r="G51" s="0">
         <v>1000</v>
       </c>
@@ -3144,7 +3127,7 @@
       </c>
       <c r="V51" s="0"/>
       <c r="W51" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C51="","Missing blog title",""),IF(E51="","Missing slides per post",""),IF(OR(E51&lt;1,E51&gt;10),"Slides per post must be 1-10",""),IF(F51="","Missing URL",""),IF(G51="","Missing width",""),IF(H51="","Missing height",""),IF(I51="","Missing theme",""),IF(M51="","Missing hero type",""),IF(N51="","Missing image direction",""),IF(U51="","Missing status",""),IF(AND(J51="Custom",K51=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C51="","Missing blog title",""),IF(E51="","Missing URL",""),IF(F51="","Missing number of slides",""),IF(OR(F51&lt;1,F51&gt;10),"Number of slides must be 1-10",""),IF(G51="","Missing width",""),IF(H51="","Missing height",""),IF(I51="","Missing theme",""),IF(M51="","Missing hero type",""),IF(N51="","Missing image direction",""),IF(U51="","Missing status",""),IF(AND(J51="Custom",K51=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="52">
@@ -3154,10 +3137,10 @@
       <c r="B52" s="0"/>
       <c r="C52" s="0"/>
       <c r="D52" s="0"/>
-      <c r="E52" s="0">
-        <v>1</v>
-      </c>
-      <c r="F52" s="0"/>
+      <c r="E52" s="0"/>
+      <c r="F52" s="0">
+        <v>1</v>
+      </c>
       <c r="G52" s="0">
         <v>1000</v>
       </c>
@@ -3199,7 +3182,7 @@
       </c>
       <c r="V52" s="0"/>
       <c r="W52" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C52="","Missing blog title",""),IF(E52="","Missing slides per post",""),IF(OR(E52&lt;1,E52&gt;10),"Slides per post must be 1-10",""),IF(F52="","Missing URL",""),IF(G52="","Missing width",""),IF(H52="","Missing height",""),IF(I52="","Missing theme",""),IF(M52="","Missing hero type",""),IF(N52="","Missing image direction",""),IF(U52="","Missing status",""),IF(AND(J52="Custom",K52=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C52="","Missing blog title",""),IF(E52="","Missing URL",""),IF(F52="","Missing number of slides",""),IF(OR(F52&lt;1,F52&gt;10),"Number of slides must be 1-10",""),IF(G52="","Missing width",""),IF(H52="","Missing height",""),IF(I52="","Missing theme",""),IF(M52="","Missing hero type",""),IF(N52="","Missing image direction",""),IF(U52="","Missing status",""),IF(AND(J52="Custom",K52=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="53">
@@ -3209,10 +3192,10 @@
       <c r="B53" s="0"/>
       <c r="C53" s="0"/>
       <c r="D53" s="0"/>
-      <c r="E53" s="0">
-        <v>1</v>
-      </c>
-      <c r="F53" s="0"/>
+      <c r="E53" s="0"/>
+      <c r="F53" s="0">
+        <v>1</v>
+      </c>
       <c r="G53" s="0">
         <v>1000</v>
       </c>
@@ -3254,7 +3237,7 @@
       </c>
       <c r="V53" s="0"/>
       <c r="W53" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C53="","Missing blog title",""),IF(E53="","Missing slides per post",""),IF(OR(E53&lt;1,E53&gt;10),"Slides per post must be 1-10",""),IF(F53="","Missing URL",""),IF(G53="","Missing width",""),IF(H53="","Missing height",""),IF(I53="","Missing theme",""),IF(M53="","Missing hero type",""),IF(N53="","Missing image direction",""),IF(U53="","Missing status",""),IF(AND(J53="Custom",K53=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C53="","Missing blog title",""),IF(E53="","Missing URL",""),IF(F53="","Missing number of slides",""),IF(OR(F53&lt;1,F53&gt;10),"Number of slides must be 1-10",""),IF(G53="","Missing width",""),IF(H53="","Missing height",""),IF(I53="","Missing theme",""),IF(M53="","Missing hero type",""),IF(N53="","Missing image direction",""),IF(U53="","Missing status",""),IF(AND(J53="Custom",K53=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="54">
@@ -3264,10 +3247,10 @@
       <c r="B54" s="0"/>
       <c r="C54" s="0"/>
       <c r="D54" s="0"/>
-      <c r="E54" s="0">
-        <v>1</v>
-      </c>
-      <c r="F54" s="0"/>
+      <c r="E54" s="0"/>
+      <c r="F54" s="0">
+        <v>1</v>
+      </c>
       <c r="G54" s="0">
         <v>1000</v>
       </c>
@@ -3309,7 +3292,7 @@
       </c>
       <c r="V54" s="0"/>
       <c r="W54" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C54="","Missing blog title",""),IF(E54="","Missing slides per post",""),IF(OR(E54&lt;1,E54&gt;10),"Slides per post must be 1-10",""),IF(F54="","Missing URL",""),IF(G54="","Missing width",""),IF(H54="","Missing height",""),IF(I54="","Missing theme",""),IF(M54="","Missing hero type",""),IF(N54="","Missing image direction",""),IF(U54="","Missing status",""),IF(AND(J54="Custom",K54=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C54="","Missing blog title",""),IF(E54="","Missing URL",""),IF(F54="","Missing number of slides",""),IF(OR(F54&lt;1,F54&gt;10),"Number of slides must be 1-10",""),IF(G54="","Missing width",""),IF(H54="","Missing height",""),IF(I54="","Missing theme",""),IF(M54="","Missing hero type",""),IF(N54="","Missing image direction",""),IF(U54="","Missing status",""),IF(AND(J54="Custom",K54=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="55">
@@ -3319,10 +3302,10 @@
       <c r="B55" s="0"/>
       <c r="C55" s="0"/>
       <c r="D55" s="0"/>
-      <c r="E55" s="0">
-        <v>1</v>
-      </c>
-      <c r="F55" s="0"/>
+      <c r="E55" s="0"/>
+      <c r="F55" s="0">
+        <v>1</v>
+      </c>
       <c r="G55" s="0">
         <v>1000</v>
       </c>
@@ -3364,7 +3347,7 @@
       </c>
       <c r="V55" s="0"/>
       <c r="W55" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C55="","Missing blog title",""),IF(E55="","Missing slides per post",""),IF(OR(E55&lt;1,E55&gt;10),"Slides per post must be 1-10",""),IF(F55="","Missing URL",""),IF(G55="","Missing width",""),IF(H55="","Missing height",""),IF(I55="","Missing theme",""),IF(M55="","Missing hero type",""),IF(N55="","Missing image direction",""),IF(U55="","Missing status",""),IF(AND(J55="Custom",K55=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C55="","Missing blog title",""),IF(E55="","Missing URL",""),IF(F55="","Missing number of slides",""),IF(OR(F55&lt;1,F55&gt;10),"Number of slides must be 1-10",""),IF(G55="","Missing width",""),IF(H55="","Missing height",""),IF(I55="","Missing theme",""),IF(M55="","Missing hero type",""),IF(N55="","Missing image direction",""),IF(U55="","Missing status",""),IF(AND(J55="Custom",K55=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="56">
@@ -3374,10 +3357,10 @@
       <c r="B56" s="0"/>
       <c r="C56" s="0"/>
       <c r="D56" s="0"/>
-      <c r="E56" s="0">
-        <v>1</v>
-      </c>
-      <c r="F56" s="0"/>
+      <c r="E56" s="0"/>
+      <c r="F56" s="0">
+        <v>1</v>
+      </c>
       <c r="G56" s="0">
         <v>1000</v>
       </c>
@@ -3419,7 +3402,7 @@
       </c>
       <c r="V56" s="0"/>
       <c r="W56" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C56="","Missing blog title",""),IF(E56="","Missing slides per post",""),IF(OR(E56&lt;1,E56&gt;10),"Slides per post must be 1-10",""),IF(F56="","Missing URL",""),IF(G56="","Missing width",""),IF(H56="","Missing height",""),IF(I56="","Missing theme",""),IF(M56="","Missing hero type",""),IF(N56="","Missing image direction",""),IF(U56="","Missing status",""),IF(AND(J56="Custom",K56=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C56="","Missing blog title",""),IF(E56="","Missing URL",""),IF(F56="","Missing number of slides",""),IF(OR(F56&lt;1,F56&gt;10),"Number of slides must be 1-10",""),IF(G56="","Missing width",""),IF(H56="","Missing height",""),IF(I56="","Missing theme",""),IF(M56="","Missing hero type",""),IF(N56="","Missing image direction",""),IF(U56="","Missing status",""),IF(AND(J56="Custom",K56=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="57">
@@ -3429,10 +3412,10 @@
       <c r="B57" s="0"/>
       <c r="C57" s="0"/>
       <c r="D57" s="0"/>
-      <c r="E57" s="0">
-        <v>1</v>
-      </c>
-      <c r="F57" s="0"/>
+      <c r="E57" s="0"/>
+      <c r="F57" s="0">
+        <v>1</v>
+      </c>
       <c r="G57" s="0">
         <v>1000</v>
       </c>
@@ -3474,7 +3457,7 @@
       </c>
       <c r="V57" s="0"/>
       <c r="W57" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C57="","Missing blog title",""),IF(E57="","Missing slides per post",""),IF(OR(E57&lt;1,E57&gt;10),"Slides per post must be 1-10",""),IF(F57="","Missing URL",""),IF(G57="","Missing width",""),IF(H57="","Missing height",""),IF(I57="","Missing theme",""),IF(M57="","Missing hero type",""),IF(N57="","Missing image direction",""),IF(U57="","Missing status",""),IF(AND(J57="Custom",K57=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C57="","Missing blog title",""),IF(E57="","Missing URL",""),IF(F57="","Missing number of slides",""),IF(OR(F57&lt;1,F57&gt;10),"Number of slides must be 1-10",""),IF(G57="","Missing width",""),IF(H57="","Missing height",""),IF(I57="","Missing theme",""),IF(M57="","Missing hero type",""),IF(N57="","Missing image direction",""),IF(U57="","Missing status",""),IF(AND(J57="Custom",K57=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="58">
@@ -3484,10 +3467,10 @@
       <c r="B58" s="0"/>
       <c r="C58" s="0"/>
       <c r="D58" s="0"/>
-      <c r="E58" s="0">
-        <v>1</v>
-      </c>
-      <c r="F58" s="0"/>
+      <c r="E58" s="0"/>
+      <c r="F58" s="0">
+        <v>1</v>
+      </c>
       <c r="G58" s="0">
         <v>1000</v>
       </c>
@@ -3529,7 +3512,7 @@
       </c>
       <c r="V58" s="0"/>
       <c r="W58" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C58="","Missing blog title",""),IF(E58="","Missing slides per post",""),IF(OR(E58&lt;1,E58&gt;10),"Slides per post must be 1-10",""),IF(F58="","Missing URL",""),IF(G58="","Missing width",""),IF(H58="","Missing height",""),IF(I58="","Missing theme",""),IF(M58="","Missing hero type",""),IF(N58="","Missing image direction",""),IF(U58="","Missing status",""),IF(AND(J58="Custom",K58=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C58="","Missing blog title",""),IF(E58="","Missing URL",""),IF(F58="","Missing number of slides",""),IF(OR(F58&lt;1,F58&gt;10),"Number of slides must be 1-10",""),IF(G58="","Missing width",""),IF(H58="","Missing height",""),IF(I58="","Missing theme",""),IF(M58="","Missing hero type",""),IF(N58="","Missing image direction",""),IF(U58="","Missing status",""),IF(AND(J58="Custom",K58=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="59">
@@ -3539,10 +3522,10 @@
       <c r="B59" s="0"/>
       <c r="C59" s="0"/>
       <c r="D59" s="0"/>
-      <c r="E59" s="0">
-        <v>1</v>
-      </c>
-      <c r="F59" s="0"/>
+      <c r="E59" s="0"/>
+      <c r="F59" s="0">
+        <v>1</v>
+      </c>
       <c r="G59" s="0">
         <v>1000</v>
       </c>
@@ -3584,7 +3567,7 @@
       </c>
       <c r="V59" s="0"/>
       <c r="W59" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C59="","Missing blog title",""),IF(E59="","Missing slides per post",""),IF(OR(E59&lt;1,E59&gt;10),"Slides per post must be 1-10",""),IF(F59="","Missing URL",""),IF(G59="","Missing width",""),IF(H59="","Missing height",""),IF(I59="","Missing theme",""),IF(M59="","Missing hero type",""),IF(N59="","Missing image direction",""),IF(U59="","Missing status",""),IF(AND(J59="Custom",K59=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C59="","Missing blog title",""),IF(E59="","Missing URL",""),IF(F59="","Missing number of slides",""),IF(OR(F59&lt;1,F59&gt;10),"Number of slides must be 1-10",""),IF(G59="","Missing width",""),IF(H59="","Missing height",""),IF(I59="","Missing theme",""),IF(M59="","Missing hero type",""),IF(N59="","Missing image direction",""),IF(U59="","Missing status",""),IF(AND(J59="Custom",K59=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="60">
@@ -3594,10 +3577,10 @@
       <c r="B60" s="0"/>
       <c r="C60" s="0"/>
       <c r="D60" s="0"/>
-      <c r="E60" s="0">
-        <v>1</v>
-      </c>
-      <c r="F60" s="0"/>
+      <c r="E60" s="0"/>
+      <c r="F60" s="0">
+        <v>1</v>
+      </c>
       <c r="G60" s="0">
         <v>1000</v>
       </c>
@@ -3639,7 +3622,7 @@
       </c>
       <c r="V60" s="0"/>
       <c r="W60" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C60="","Missing blog title",""),IF(E60="","Missing slides per post",""),IF(OR(E60&lt;1,E60&gt;10),"Slides per post must be 1-10",""),IF(F60="","Missing URL",""),IF(G60="","Missing width",""),IF(H60="","Missing height",""),IF(I60="","Missing theme",""),IF(M60="","Missing hero type",""),IF(N60="","Missing image direction",""),IF(U60="","Missing status",""),IF(AND(J60="Custom",K60=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C60="","Missing blog title",""),IF(E60="","Missing URL",""),IF(F60="","Missing number of slides",""),IF(OR(F60&lt;1,F60&gt;10),"Number of slides must be 1-10",""),IF(G60="","Missing width",""),IF(H60="","Missing height",""),IF(I60="","Missing theme",""),IF(M60="","Missing hero type",""),IF(N60="","Missing image direction",""),IF(U60="","Missing status",""),IF(AND(J60="Custom",K60=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="61">
@@ -3649,10 +3632,10 @@
       <c r="B61" s="0"/>
       <c r="C61" s="0"/>
       <c r="D61" s="0"/>
-      <c r="E61" s="0">
-        <v>1</v>
-      </c>
-      <c r="F61" s="0"/>
+      <c r="E61" s="0"/>
+      <c r="F61" s="0">
+        <v>1</v>
+      </c>
       <c r="G61" s="0">
         <v>1000</v>
       </c>
@@ -3694,7 +3677,7 @@
       </c>
       <c r="V61" s="0"/>
       <c r="W61" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C61="","Missing blog title",""),IF(E61="","Missing slides per post",""),IF(OR(E61&lt;1,E61&gt;10),"Slides per post must be 1-10",""),IF(F61="","Missing URL",""),IF(G61="","Missing width",""),IF(H61="","Missing height",""),IF(I61="","Missing theme",""),IF(M61="","Missing hero type",""),IF(N61="","Missing image direction",""),IF(U61="","Missing status",""),IF(AND(J61="Custom",K61=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C61="","Missing blog title",""),IF(E61="","Missing URL",""),IF(F61="","Missing number of slides",""),IF(OR(F61&lt;1,F61&gt;10),"Number of slides must be 1-10",""),IF(G61="","Missing width",""),IF(H61="","Missing height",""),IF(I61="","Missing theme",""),IF(M61="","Missing hero type",""),IF(N61="","Missing image direction",""),IF(U61="","Missing status",""),IF(AND(J61="Custom",K61=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="62">
@@ -3704,10 +3687,10 @@
       <c r="B62" s="0"/>
       <c r="C62" s="0"/>
       <c r="D62" s="0"/>
-      <c r="E62" s="0">
-        <v>1</v>
-      </c>
-      <c r="F62" s="0"/>
+      <c r="E62" s="0"/>
+      <c r="F62" s="0">
+        <v>1</v>
+      </c>
       <c r="G62" s="0">
         <v>1000</v>
       </c>
@@ -3749,7 +3732,7 @@
       </c>
       <c r="V62" s="0"/>
       <c r="W62" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C62="","Missing blog title",""),IF(E62="","Missing slides per post",""),IF(OR(E62&lt;1,E62&gt;10),"Slides per post must be 1-10",""),IF(F62="","Missing URL",""),IF(G62="","Missing width",""),IF(H62="","Missing height",""),IF(I62="","Missing theme",""),IF(M62="","Missing hero type",""),IF(N62="","Missing image direction",""),IF(U62="","Missing status",""),IF(AND(J62="Custom",K62=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C62="","Missing blog title",""),IF(E62="","Missing URL",""),IF(F62="","Missing number of slides",""),IF(OR(F62&lt;1,F62&gt;10),"Number of slides must be 1-10",""),IF(G62="","Missing width",""),IF(H62="","Missing height",""),IF(I62="","Missing theme",""),IF(M62="","Missing hero type",""),IF(N62="","Missing image direction",""),IF(U62="","Missing status",""),IF(AND(J62="Custom",K62=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="63">
@@ -3759,10 +3742,10 @@
       <c r="B63" s="0"/>
       <c r="C63" s="0"/>
       <c r="D63" s="0"/>
-      <c r="E63" s="0">
-        <v>1</v>
-      </c>
-      <c r="F63" s="0"/>
+      <c r="E63" s="0"/>
+      <c r="F63" s="0">
+        <v>1</v>
+      </c>
       <c r="G63" s="0">
         <v>1000</v>
       </c>
@@ -3804,7 +3787,7 @@
       </c>
       <c r="V63" s="0"/>
       <c r="W63" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C63="","Missing blog title",""),IF(E63="","Missing slides per post",""),IF(OR(E63&lt;1,E63&gt;10),"Slides per post must be 1-10",""),IF(F63="","Missing URL",""),IF(G63="","Missing width",""),IF(H63="","Missing height",""),IF(I63="","Missing theme",""),IF(M63="","Missing hero type",""),IF(N63="","Missing image direction",""),IF(U63="","Missing status",""),IF(AND(J63="Custom",K63=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C63="","Missing blog title",""),IF(E63="","Missing URL",""),IF(F63="","Missing number of slides",""),IF(OR(F63&lt;1,F63&gt;10),"Number of slides must be 1-10",""),IF(G63="","Missing width",""),IF(H63="","Missing height",""),IF(I63="","Missing theme",""),IF(M63="","Missing hero type",""),IF(N63="","Missing image direction",""),IF(U63="","Missing status",""),IF(AND(J63="Custom",K63=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="64">
@@ -3814,10 +3797,10 @@
       <c r="B64" s="0"/>
       <c r="C64" s="0"/>
       <c r="D64" s="0"/>
-      <c r="E64" s="0">
-        <v>1</v>
-      </c>
-      <c r="F64" s="0"/>
+      <c r="E64" s="0"/>
+      <c r="F64" s="0">
+        <v>1</v>
+      </c>
       <c r="G64" s="0">
         <v>1000</v>
       </c>
@@ -3859,7 +3842,7 @@
       </c>
       <c r="V64" s="0"/>
       <c r="W64" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C64="","Missing blog title",""),IF(E64="","Missing slides per post",""),IF(OR(E64&lt;1,E64&gt;10),"Slides per post must be 1-10",""),IF(F64="","Missing URL",""),IF(G64="","Missing width",""),IF(H64="","Missing height",""),IF(I64="","Missing theme",""),IF(M64="","Missing hero type",""),IF(N64="","Missing image direction",""),IF(U64="","Missing status",""),IF(AND(J64="Custom",K64=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C64="","Missing blog title",""),IF(E64="","Missing URL",""),IF(F64="","Missing number of slides",""),IF(OR(F64&lt;1,F64&gt;10),"Number of slides must be 1-10",""),IF(G64="","Missing width",""),IF(H64="","Missing height",""),IF(I64="","Missing theme",""),IF(M64="","Missing hero type",""),IF(N64="","Missing image direction",""),IF(U64="","Missing status",""),IF(AND(J64="Custom",K64=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="65">
@@ -3869,10 +3852,10 @@
       <c r="B65" s="0"/>
       <c r="C65" s="0"/>
       <c r="D65" s="0"/>
-      <c r="E65" s="0">
-        <v>1</v>
-      </c>
-      <c r="F65" s="0"/>
+      <c r="E65" s="0"/>
+      <c r="F65" s="0">
+        <v>1</v>
+      </c>
       <c r="G65" s="0">
         <v>1000</v>
       </c>
@@ -3914,7 +3897,7 @@
       </c>
       <c r="V65" s="0"/>
       <c r="W65" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C65="","Missing blog title",""),IF(E65="","Missing slides per post",""),IF(OR(E65&lt;1,E65&gt;10),"Slides per post must be 1-10",""),IF(F65="","Missing URL",""),IF(G65="","Missing width",""),IF(H65="","Missing height",""),IF(I65="","Missing theme",""),IF(M65="","Missing hero type",""),IF(N65="","Missing image direction",""),IF(U65="","Missing status",""),IF(AND(J65="Custom",K65=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C65="","Missing blog title",""),IF(E65="","Missing URL",""),IF(F65="","Missing number of slides",""),IF(OR(F65&lt;1,F65&gt;10),"Number of slides must be 1-10",""),IF(G65="","Missing width",""),IF(H65="","Missing height",""),IF(I65="","Missing theme",""),IF(M65="","Missing hero type",""),IF(N65="","Missing image direction",""),IF(U65="","Missing status",""),IF(AND(J65="Custom",K65=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="66">
@@ -3924,10 +3907,10 @@
       <c r="B66" s="0"/>
       <c r="C66" s="0"/>
       <c r="D66" s="0"/>
-      <c r="E66" s="0">
-        <v>1</v>
-      </c>
-      <c r="F66" s="0"/>
+      <c r="E66" s="0"/>
+      <c r="F66" s="0">
+        <v>1</v>
+      </c>
       <c r="G66" s="0">
         <v>1000</v>
       </c>
@@ -3969,7 +3952,7 @@
       </c>
       <c r="V66" s="0"/>
       <c r="W66" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C66="","Missing blog title",""),IF(E66="","Missing slides per post",""),IF(OR(E66&lt;1,E66&gt;10),"Slides per post must be 1-10",""),IF(F66="","Missing URL",""),IF(G66="","Missing width",""),IF(H66="","Missing height",""),IF(I66="","Missing theme",""),IF(M66="","Missing hero type",""),IF(N66="","Missing image direction",""),IF(U66="","Missing status",""),IF(AND(J66="Custom",K66=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C66="","Missing blog title",""),IF(E66="","Missing URL",""),IF(F66="","Missing number of slides",""),IF(OR(F66&lt;1,F66&gt;10),"Number of slides must be 1-10",""),IF(G66="","Missing width",""),IF(H66="","Missing height",""),IF(I66="","Missing theme",""),IF(M66="","Missing hero type",""),IF(N66="","Missing image direction",""),IF(U66="","Missing status",""),IF(AND(J66="Custom",K66=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="67">
@@ -3979,10 +3962,10 @@
       <c r="B67" s="0"/>
       <c r="C67" s="0"/>
       <c r="D67" s="0"/>
-      <c r="E67" s="0">
-        <v>1</v>
-      </c>
-      <c r="F67" s="0"/>
+      <c r="E67" s="0"/>
+      <c r="F67" s="0">
+        <v>1</v>
+      </c>
       <c r="G67" s="0">
         <v>1000</v>
       </c>
@@ -4024,7 +4007,7 @@
       </c>
       <c r="V67" s="0"/>
       <c r="W67" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C67="","Missing blog title",""),IF(E67="","Missing slides per post",""),IF(OR(E67&lt;1,E67&gt;10),"Slides per post must be 1-10",""),IF(F67="","Missing URL",""),IF(G67="","Missing width",""),IF(H67="","Missing height",""),IF(I67="","Missing theme",""),IF(M67="","Missing hero type",""),IF(N67="","Missing image direction",""),IF(U67="","Missing status",""),IF(AND(J67="Custom",K67=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C67="","Missing blog title",""),IF(E67="","Missing URL",""),IF(F67="","Missing number of slides",""),IF(OR(F67&lt;1,F67&gt;10),"Number of slides must be 1-10",""),IF(G67="","Missing width",""),IF(H67="","Missing height",""),IF(I67="","Missing theme",""),IF(M67="","Missing hero type",""),IF(N67="","Missing image direction",""),IF(U67="","Missing status",""),IF(AND(J67="Custom",K67=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="68">
@@ -4034,10 +4017,10 @@
       <c r="B68" s="0"/>
       <c r="C68" s="0"/>
       <c r="D68" s="0"/>
-      <c r="E68" s="0">
-        <v>1</v>
-      </c>
-      <c r="F68" s="0"/>
+      <c r="E68" s="0"/>
+      <c r="F68" s="0">
+        <v>1</v>
+      </c>
       <c r="G68" s="0">
         <v>1000</v>
       </c>
@@ -4079,7 +4062,7 @@
       </c>
       <c r="V68" s="0"/>
       <c r="W68" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C68="","Missing blog title",""),IF(E68="","Missing slides per post",""),IF(OR(E68&lt;1,E68&gt;10),"Slides per post must be 1-10",""),IF(F68="","Missing URL",""),IF(G68="","Missing width",""),IF(H68="","Missing height",""),IF(I68="","Missing theme",""),IF(M68="","Missing hero type",""),IF(N68="","Missing image direction",""),IF(U68="","Missing status",""),IF(AND(J68="Custom",K68=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C68="","Missing blog title",""),IF(E68="","Missing URL",""),IF(F68="","Missing number of slides",""),IF(OR(F68&lt;1,F68&gt;10),"Number of slides must be 1-10",""),IF(G68="","Missing width",""),IF(H68="","Missing height",""),IF(I68="","Missing theme",""),IF(M68="","Missing hero type",""),IF(N68="","Missing image direction",""),IF(U68="","Missing status",""),IF(AND(J68="Custom",K68=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="69">
@@ -4089,10 +4072,10 @@
       <c r="B69" s="0"/>
       <c r="C69" s="0"/>
       <c r="D69" s="0"/>
-      <c r="E69" s="0">
-        <v>1</v>
-      </c>
-      <c r="F69" s="0"/>
+      <c r="E69" s="0"/>
+      <c r="F69" s="0">
+        <v>1</v>
+      </c>
       <c r="G69" s="0">
         <v>1000</v>
       </c>
@@ -4134,7 +4117,7 @@
       </c>
       <c r="V69" s="0"/>
       <c r="W69" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C69="","Missing blog title",""),IF(E69="","Missing slides per post",""),IF(OR(E69&lt;1,E69&gt;10),"Slides per post must be 1-10",""),IF(F69="","Missing URL",""),IF(G69="","Missing width",""),IF(H69="","Missing height",""),IF(I69="","Missing theme",""),IF(M69="","Missing hero type",""),IF(N69="","Missing image direction",""),IF(U69="","Missing status",""),IF(AND(J69="Custom",K69=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C69="","Missing blog title",""),IF(E69="","Missing URL",""),IF(F69="","Missing number of slides",""),IF(OR(F69&lt;1,F69&gt;10),"Number of slides must be 1-10",""),IF(G69="","Missing width",""),IF(H69="","Missing height",""),IF(I69="","Missing theme",""),IF(M69="","Missing hero type",""),IF(N69="","Missing image direction",""),IF(U69="","Missing status",""),IF(AND(J69="Custom",K69=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="70">
@@ -4144,10 +4127,10 @@
       <c r="B70" s="0"/>
       <c r="C70" s="0"/>
       <c r="D70" s="0"/>
-      <c r="E70" s="0">
-        <v>1</v>
-      </c>
-      <c r="F70" s="0"/>
+      <c r="E70" s="0"/>
+      <c r="F70" s="0">
+        <v>1</v>
+      </c>
       <c r="G70" s="0">
         <v>1000</v>
       </c>
@@ -4189,7 +4172,7 @@
       </c>
       <c r="V70" s="0"/>
       <c r="W70" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C70="","Missing blog title",""),IF(E70="","Missing slides per post",""),IF(OR(E70&lt;1,E70&gt;10),"Slides per post must be 1-10",""),IF(F70="","Missing URL",""),IF(G70="","Missing width",""),IF(H70="","Missing height",""),IF(I70="","Missing theme",""),IF(M70="","Missing hero type",""),IF(N70="","Missing image direction",""),IF(U70="","Missing status",""),IF(AND(J70="Custom",K70=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C70="","Missing blog title",""),IF(E70="","Missing URL",""),IF(F70="","Missing number of slides",""),IF(OR(F70&lt;1,F70&gt;10),"Number of slides must be 1-10",""),IF(G70="","Missing width",""),IF(H70="","Missing height",""),IF(I70="","Missing theme",""),IF(M70="","Missing hero type",""),IF(N70="","Missing image direction",""),IF(U70="","Missing status",""),IF(AND(J70="Custom",K70=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="71">
@@ -4199,10 +4182,10 @@
       <c r="B71" s="0"/>
       <c r="C71" s="0"/>
       <c r="D71" s="0"/>
-      <c r="E71" s="0">
-        <v>1</v>
-      </c>
-      <c r="F71" s="0"/>
+      <c r="E71" s="0"/>
+      <c r="F71" s="0">
+        <v>1</v>
+      </c>
       <c r="G71" s="0">
         <v>1000</v>
       </c>
@@ -4244,7 +4227,7 @@
       </c>
       <c r="V71" s="0"/>
       <c r="W71" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C71="","Missing blog title",""),IF(E71="","Missing slides per post",""),IF(OR(E71&lt;1,E71&gt;10),"Slides per post must be 1-10",""),IF(F71="","Missing URL",""),IF(G71="","Missing width",""),IF(H71="","Missing height",""),IF(I71="","Missing theme",""),IF(M71="","Missing hero type",""),IF(N71="","Missing image direction",""),IF(U71="","Missing status",""),IF(AND(J71="Custom",K71=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C71="","Missing blog title",""),IF(E71="","Missing URL",""),IF(F71="","Missing number of slides",""),IF(OR(F71&lt;1,F71&gt;10),"Number of slides must be 1-10",""),IF(G71="","Missing width",""),IF(H71="","Missing height",""),IF(I71="","Missing theme",""),IF(M71="","Missing hero type",""),IF(N71="","Missing image direction",""),IF(U71="","Missing status",""),IF(AND(J71="Custom",K71=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="72">
@@ -4254,10 +4237,10 @@
       <c r="B72" s="0"/>
       <c r="C72" s="0"/>
       <c r="D72" s="0"/>
-      <c r="E72" s="0">
-        <v>1</v>
-      </c>
-      <c r="F72" s="0"/>
+      <c r="E72" s="0"/>
+      <c r="F72" s="0">
+        <v>1</v>
+      </c>
       <c r="G72" s="0">
         <v>1000</v>
       </c>
@@ -4299,7 +4282,7 @@
       </c>
       <c r="V72" s="0"/>
       <c r="W72" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C72="","Missing blog title",""),IF(E72="","Missing slides per post",""),IF(OR(E72&lt;1,E72&gt;10),"Slides per post must be 1-10",""),IF(F72="","Missing URL",""),IF(G72="","Missing width",""),IF(H72="","Missing height",""),IF(I72="","Missing theme",""),IF(M72="","Missing hero type",""),IF(N72="","Missing image direction",""),IF(U72="","Missing status",""),IF(AND(J72="Custom",K72=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C72="","Missing blog title",""),IF(E72="","Missing URL",""),IF(F72="","Missing number of slides",""),IF(OR(F72&lt;1,F72&gt;10),"Number of slides must be 1-10",""),IF(G72="","Missing width",""),IF(H72="","Missing height",""),IF(I72="","Missing theme",""),IF(M72="","Missing hero type",""),IF(N72="","Missing image direction",""),IF(U72="","Missing status",""),IF(AND(J72="Custom",K72=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="73">
@@ -4309,10 +4292,10 @@
       <c r="B73" s="0"/>
       <c r="C73" s="0"/>
       <c r="D73" s="0"/>
-      <c r="E73" s="0">
-        <v>1</v>
-      </c>
-      <c r="F73" s="0"/>
+      <c r="E73" s="0"/>
+      <c r="F73" s="0">
+        <v>1</v>
+      </c>
       <c r="G73" s="0">
         <v>1000</v>
       </c>
@@ -4354,7 +4337,7 @@
       </c>
       <c r="V73" s="0"/>
       <c r="W73" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C73="","Missing blog title",""),IF(E73="","Missing slides per post",""),IF(OR(E73&lt;1,E73&gt;10),"Slides per post must be 1-10",""),IF(F73="","Missing URL",""),IF(G73="","Missing width",""),IF(H73="","Missing height",""),IF(I73="","Missing theme",""),IF(M73="","Missing hero type",""),IF(N73="","Missing image direction",""),IF(U73="","Missing status",""),IF(AND(J73="Custom",K73=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C73="","Missing blog title",""),IF(E73="","Missing URL",""),IF(F73="","Missing number of slides",""),IF(OR(F73&lt;1,F73&gt;10),"Number of slides must be 1-10",""),IF(G73="","Missing width",""),IF(H73="","Missing height",""),IF(I73="","Missing theme",""),IF(M73="","Missing hero type",""),IF(N73="","Missing image direction",""),IF(U73="","Missing status",""),IF(AND(J73="Custom",K73=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="74">
@@ -4364,10 +4347,10 @@
       <c r="B74" s="0"/>
       <c r="C74" s="0"/>
       <c r="D74" s="0"/>
-      <c r="E74" s="0">
-        <v>1</v>
-      </c>
-      <c r="F74" s="0"/>
+      <c r="E74" s="0"/>
+      <c r="F74" s="0">
+        <v>1</v>
+      </c>
       <c r="G74" s="0">
         <v>1000</v>
       </c>
@@ -4409,7 +4392,7 @@
       </c>
       <c r="V74" s="0"/>
       <c r="W74" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C74="","Missing blog title",""),IF(E74="","Missing slides per post",""),IF(OR(E74&lt;1,E74&gt;10),"Slides per post must be 1-10",""),IF(F74="","Missing URL",""),IF(G74="","Missing width",""),IF(H74="","Missing height",""),IF(I74="","Missing theme",""),IF(M74="","Missing hero type",""),IF(N74="","Missing image direction",""),IF(U74="","Missing status",""),IF(AND(J74="Custom",K74=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C74="","Missing blog title",""),IF(E74="","Missing URL",""),IF(F74="","Missing number of slides",""),IF(OR(F74&lt;1,F74&gt;10),"Number of slides must be 1-10",""),IF(G74="","Missing width",""),IF(H74="","Missing height",""),IF(I74="","Missing theme",""),IF(M74="","Missing hero type",""),IF(N74="","Missing image direction",""),IF(U74="","Missing status",""),IF(AND(J74="Custom",K74=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="75">
@@ -4419,10 +4402,10 @@
       <c r="B75" s="0"/>
       <c r="C75" s="0"/>
       <c r="D75" s="0"/>
-      <c r="E75" s="0">
-        <v>1</v>
-      </c>
-      <c r="F75" s="0"/>
+      <c r="E75" s="0"/>
+      <c r="F75" s="0">
+        <v>1</v>
+      </c>
       <c r="G75" s="0">
         <v>1000</v>
       </c>
@@ -4464,7 +4447,7 @@
       </c>
       <c r="V75" s="0"/>
       <c r="W75" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C75="","Missing blog title",""),IF(E75="","Missing slides per post",""),IF(OR(E75&lt;1,E75&gt;10),"Slides per post must be 1-10",""),IF(F75="","Missing URL",""),IF(G75="","Missing width",""),IF(H75="","Missing height",""),IF(I75="","Missing theme",""),IF(M75="","Missing hero type",""),IF(N75="","Missing image direction",""),IF(U75="","Missing status",""),IF(AND(J75="Custom",K75=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C75="","Missing blog title",""),IF(E75="","Missing URL",""),IF(F75="","Missing number of slides",""),IF(OR(F75&lt;1,F75&gt;10),"Number of slides must be 1-10",""),IF(G75="","Missing width",""),IF(H75="","Missing height",""),IF(I75="","Missing theme",""),IF(M75="","Missing hero type",""),IF(N75="","Missing image direction",""),IF(U75="","Missing status",""),IF(AND(J75="Custom",K75=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="76">
@@ -4474,10 +4457,10 @@
       <c r="B76" s="0"/>
       <c r="C76" s="0"/>
       <c r="D76" s="0"/>
-      <c r="E76" s="0">
-        <v>1</v>
-      </c>
-      <c r="F76" s="0"/>
+      <c r="E76" s="0"/>
+      <c r="F76" s="0">
+        <v>1</v>
+      </c>
       <c r="G76" s="0">
         <v>1000</v>
       </c>
@@ -4519,7 +4502,7 @@
       </c>
       <c r="V76" s="0"/>
       <c r="W76" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C76="","Missing blog title",""),IF(E76="","Missing slides per post",""),IF(OR(E76&lt;1,E76&gt;10),"Slides per post must be 1-10",""),IF(F76="","Missing URL",""),IF(G76="","Missing width",""),IF(H76="","Missing height",""),IF(I76="","Missing theme",""),IF(M76="","Missing hero type",""),IF(N76="","Missing image direction",""),IF(U76="","Missing status",""),IF(AND(J76="Custom",K76=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C76="","Missing blog title",""),IF(E76="","Missing URL",""),IF(F76="","Missing number of slides",""),IF(OR(F76&lt;1,F76&gt;10),"Number of slides must be 1-10",""),IF(G76="","Missing width",""),IF(H76="","Missing height",""),IF(I76="","Missing theme",""),IF(M76="","Missing hero type",""),IF(N76="","Missing image direction",""),IF(U76="","Missing status",""),IF(AND(J76="Custom",K76=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="77">
@@ -4529,10 +4512,10 @@
       <c r="B77" s="0"/>
       <c r="C77" s="0"/>
       <c r="D77" s="0"/>
-      <c r="E77" s="0">
-        <v>1</v>
-      </c>
-      <c r="F77" s="0"/>
+      <c r="E77" s="0"/>
+      <c r="F77" s="0">
+        <v>1</v>
+      </c>
       <c r="G77" s="0">
         <v>1000</v>
       </c>
@@ -4574,7 +4557,7 @@
       </c>
       <c r="V77" s="0"/>
       <c r="W77" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C77="","Missing blog title",""),IF(E77="","Missing slides per post",""),IF(OR(E77&lt;1,E77&gt;10),"Slides per post must be 1-10",""),IF(F77="","Missing URL",""),IF(G77="","Missing width",""),IF(H77="","Missing height",""),IF(I77="","Missing theme",""),IF(M77="","Missing hero type",""),IF(N77="","Missing image direction",""),IF(U77="","Missing status",""),IF(AND(J77="Custom",K77=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C77="","Missing blog title",""),IF(E77="","Missing URL",""),IF(F77="","Missing number of slides",""),IF(OR(F77&lt;1,F77&gt;10),"Number of slides must be 1-10",""),IF(G77="","Missing width",""),IF(H77="","Missing height",""),IF(I77="","Missing theme",""),IF(M77="","Missing hero type",""),IF(N77="","Missing image direction",""),IF(U77="","Missing status",""),IF(AND(J77="Custom",K77=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="78">
@@ -4584,10 +4567,10 @@
       <c r="B78" s="0"/>
       <c r="C78" s="0"/>
       <c r="D78" s="0"/>
-      <c r="E78" s="0">
-        <v>1</v>
-      </c>
-      <c r="F78" s="0"/>
+      <c r="E78" s="0"/>
+      <c r="F78" s="0">
+        <v>1</v>
+      </c>
       <c r="G78" s="0">
         <v>1000</v>
       </c>
@@ -4629,7 +4612,7 @@
       </c>
       <c r="V78" s="0"/>
       <c r="W78" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C78="","Missing blog title",""),IF(E78="","Missing slides per post",""),IF(OR(E78&lt;1,E78&gt;10),"Slides per post must be 1-10",""),IF(F78="","Missing URL",""),IF(G78="","Missing width",""),IF(H78="","Missing height",""),IF(I78="","Missing theme",""),IF(M78="","Missing hero type",""),IF(N78="","Missing image direction",""),IF(U78="","Missing status",""),IF(AND(J78="Custom",K78=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C78="","Missing blog title",""),IF(E78="","Missing URL",""),IF(F78="","Missing number of slides",""),IF(OR(F78&lt;1,F78&gt;10),"Number of slides must be 1-10",""),IF(G78="","Missing width",""),IF(H78="","Missing height",""),IF(I78="","Missing theme",""),IF(M78="","Missing hero type",""),IF(N78="","Missing image direction",""),IF(U78="","Missing status",""),IF(AND(J78="Custom",K78=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="79">
@@ -4639,10 +4622,10 @@
       <c r="B79" s="0"/>
       <c r="C79" s="0"/>
       <c r="D79" s="0"/>
-      <c r="E79" s="0">
-        <v>1</v>
-      </c>
-      <c r="F79" s="0"/>
+      <c r="E79" s="0"/>
+      <c r="F79" s="0">
+        <v>1</v>
+      </c>
       <c r="G79" s="0">
         <v>1000</v>
       </c>
@@ -4684,7 +4667,7 @@
       </c>
       <c r="V79" s="0"/>
       <c r="W79" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C79="","Missing blog title",""),IF(E79="","Missing slides per post",""),IF(OR(E79&lt;1,E79&gt;10),"Slides per post must be 1-10",""),IF(F79="","Missing URL",""),IF(G79="","Missing width",""),IF(H79="","Missing height",""),IF(I79="","Missing theme",""),IF(M79="","Missing hero type",""),IF(N79="","Missing image direction",""),IF(U79="","Missing status",""),IF(AND(J79="Custom",K79=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C79="","Missing blog title",""),IF(E79="","Missing URL",""),IF(F79="","Missing number of slides",""),IF(OR(F79&lt;1,F79&gt;10),"Number of slides must be 1-10",""),IF(G79="","Missing width",""),IF(H79="","Missing height",""),IF(I79="","Missing theme",""),IF(M79="","Missing hero type",""),IF(N79="","Missing image direction",""),IF(U79="","Missing status",""),IF(AND(J79="Custom",K79=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="80">
@@ -4694,10 +4677,10 @@
       <c r="B80" s="0"/>
       <c r="C80" s="0"/>
       <c r="D80" s="0"/>
-      <c r="E80" s="0">
-        <v>1</v>
-      </c>
-      <c r="F80" s="0"/>
+      <c r="E80" s="0"/>
+      <c r="F80" s="0">
+        <v>1</v>
+      </c>
       <c r="G80" s="0">
         <v>1000</v>
       </c>
@@ -4739,7 +4722,7 @@
       </c>
       <c r="V80" s="0"/>
       <c r="W80" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C80="","Missing blog title",""),IF(E80="","Missing slides per post",""),IF(OR(E80&lt;1,E80&gt;10),"Slides per post must be 1-10",""),IF(F80="","Missing URL",""),IF(G80="","Missing width",""),IF(H80="","Missing height",""),IF(I80="","Missing theme",""),IF(M80="","Missing hero type",""),IF(N80="","Missing image direction",""),IF(U80="","Missing status",""),IF(AND(J80="Custom",K80=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C80="","Missing blog title",""),IF(E80="","Missing URL",""),IF(F80="","Missing number of slides",""),IF(OR(F80&lt;1,F80&gt;10),"Number of slides must be 1-10",""),IF(G80="","Missing width",""),IF(H80="","Missing height",""),IF(I80="","Missing theme",""),IF(M80="","Missing hero type",""),IF(N80="","Missing image direction",""),IF(U80="","Missing status",""),IF(AND(J80="Custom",K80=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="81">
@@ -4749,10 +4732,10 @@
       <c r="B81" s="0"/>
       <c r="C81" s="0"/>
       <c r="D81" s="0"/>
-      <c r="E81" s="0">
-        <v>1</v>
-      </c>
-      <c r="F81" s="0"/>
+      <c r="E81" s="0"/>
+      <c r="F81" s="0">
+        <v>1</v>
+      </c>
       <c r="G81" s="0">
         <v>1000</v>
       </c>
@@ -4794,7 +4777,7 @@
       </c>
       <c r="V81" s="0"/>
       <c r="W81" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C81="","Missing blog title",""),IF(E81="","Missing slides per post",""),IF(OR(E81&lt;1,E81&gt;10),"Slides per post must be 1-10",""),IF(F81="","Missing URL",""),IF(G81="","Missing width",""),IF(H81="","Missing height",""),IF(I81="","Missing theme",""),IF(M81="","Missing hero type",""),IF(N81="","Missing image direction",""),IF(U81="","Missing status",""),IF(AND(J81="Custom",K81=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C81="","Missing blog title",""),IF(E81="","Missing URL",""),IF(F81="","Missing number of slides",""),IF(OR(F81&lt;1,F81&gt;10),"Number of slides must be 1-10",""),IF(G81="","Missing width",""),IF(H81="","Missing height",""),IF(I81="","Missing theme",""),IF(M81="","Missing hero type",""),IF(N81="","Missing image direction",""),IF(U81="","Missing status",""),IF(AND(J81="Custom",K81=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="82">
@@ -4804,10 +4787,10 @@
       <c r="B82" s="0"/>
       <c r="C82" s="0"/>
       <c r="D82" s="0"/>
-      <c r="E82" s="0">
-        <v>1</v>
-      </c>
-      <c r="F82" s="0"/>
+      <c r="E82" s="0"/>
+      <c r="F82" s="0">
+        <v>1</v>
+      </c>
       <c r="G82" s="0">
         <v>1000</v>
       </c>
@@ -4849,7 +4832,7 @@
       </c>
       <c r="V82" s="0"/>
       <c r="W82" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C82="","Missing blog title",""),IF(E82="","Missing slides per post",""),IF(OR(E82&lt;1,E82&gt;10),"Slides per post must be 1-10",""),IF(F82="","Missing URL",""),IF(G82="","Missing width",""),IF(H82="","Missing height",""),IF(I82="","Missing theme",""),IF(M82="","Missing hero type",""),IF(N82="","Missing image direction",""),IF(U82="","Missing status",""),IF(AND(J82="Custom",K82=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C82="","Missing blog title",""),IF(E82="","Missing URL",""),IF(F82="","Missing number of slides",""),IF(OR(F82&lt;1,F82&gt;10),"Number of slides must be 1-10",""),IF(G82="","Missing width",""),IF(H82="","Missing height",""),IF(I82="","Missing theme",""),IF(M82="","Missing hero type",""),IF(N82="","Missing image direction",""),IF(U82="","Missing status",""),IF(AND(J82="Custom",K82=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="83">
@@ -4859,10 +4842,10 @@
       <c r="B83" s="0"/>
       <c r="C83" s="0"/>
       <c r="D83" s="0"/>
-      <c r="E83" s="0">
-        <v>1</v>
-      </c>
-      <c r="F83" s="0"/>
+      <c r="E83" s="0"/>
+      <c r="F83" s="0">
+        <v>1</v>
+      </c>
       <c r="G83" s="0">
         <v>1000</v>
       </c>
@@ -4904,7 +4887,7 @@
       </c>
       <c r="V83" s="0"/>
       <c r="W83" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C83="","Missing blog title",""),IF(E83="","Missing slides per post",""),IF(OR(E83&lt;1,E83&gt;10),"Slides per post must be 1-10",""),IF(F83="","Missing URL",""),IF(G83="","Missing width",""),IF(H83="","Missing height",""),IF(I83="","Missing theme",""),IF(M83="","Missing hero type",""),IF(N83="","Missing image direction",""),IF(U83="","Missing status",""),IF(AND(J83="Custom",K83=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C83="","Missing blog title",""),IF(E83="","Missing URL",""),IF(F83="","Missing number of slides",""),IF(OR(F83&lt;1,F83&gt;10),"Number of slides must be 1-10",""),IF(G83="","Missing width",""),IF(H83="","Missing height",""),IF(I83="","Missing theme",""),IF(M83="","Missing hero type",""),IF(N83="","Missing image direction",""),IF(U83="","Missing status",""),IF(AND(J83="Custom",K83=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="84">
@@ -4914,10 +4897,10 @@
       <c r="B84" s="0"/>
       <c r="C84" s="0"/>
       <c r="D84" s="0"/>
-      <c r="E84" s="0">
-        <v>1</v>
-      </c>
-      <c r="F84" s="0"/>
+      <c r="E84" s="0"/>
+      <c r="F84" s="0">
+        <v>1</v>
+      </c>
       <c r="G84" s="0">
         <v>1000</v>
       </c>
@@ -4959,7 +4942,7 @@
       </c>
       <c r="V84" s="0"/>
       <c r="W84" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C84="","Missing blog title",""),IF(E84="","Missing slides per post",""),IF(OR(E84&lt;1,E84&gt;10),"Slides per post must be 1-10",""),IF(F84="","Missing URL",""),IF(G84="","Missing width",""),IF(H84="","Missing height",""),IF(I84="","Missing theme",""),IF(M84="","Missing hero type",""),IF(N84="","Missing image direction",""),IF(U84="","Missing status",""),IF(AND(J84="Custom",K84=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C84="","Missing blog title",""),IF(E84="","Missing URL",""),IF(F84="","Missing number of slides",""),IF(OR(F84&lt;1,F84&gt;10),"Number of slides must be 1-10",""),IF(G84="","Missing width",""),IF(H84="","Missing height",""),IF(I84="","Missing theme",""),IF(M84="","Missing hero type",""),IF(N84="","Missing image direction",""),IF(U84="","Missing status",""),IF(AND(J84="Custom",K84=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="85">
@@ -4969,10 +4952,10 @@
       <c r="B85" s="0"/>
       <c r="C85" s="0"/>
       <c r="D85" s="0"/>
-      <c r="E85" s="0">
-        <v>1</v>
-      </c>
-      <c r="F85" s="0"/>
+      <c r="E85" s="0"/>
+      <c r="F85" s="0">
+        <v>1</v>
+      </c>
       <c r="G85" s="0">
         <v>1000</v>
       </c>
@@ -5014,7 +4997,7 @@
       </c>
       <c r="V85" s="0"/>
       <c r="W85" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C85="","Missing blog title",""),IF(E85="","Missing slides per post",""),IF(OR(E85&lt;1,E85&gt;10),"Slides per post must be 1-10",""),IF(F85="","Missing URL",""),IF(G85="","Missing width",""),IF(H85="","Missing height",""),IF(I85="","Missing theme",""),IF(M85="","Missing hero type",""),IF(N85="","Missing image direction",""),IF(U85="","Missing status",""),IF(AND(J85="Custom",K85=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C85="","Missing blog title",""),IF(E85="","Missing URL",""),IF(F85="","Missing number of slides",""),IF(OR(F85&lt;1,F85&gt;10),"Number of slides must be 1-10",""),IF(G85="","Missing width",""),IF(H85="","Missing height",""),IF(I85="","Missing theme",""),IF(M85="","Missing hero type",""),IF(N85="","Missing image direction",""),IF(U85="","Missing status",""),IF(AND(J85="Custom",K85=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="86">
@@ -5024,10 +5007,10 @@
       <c r="B86" s="0"/>
       <c r="C86" s="0"/>
       <c r="D86" s="0"/>
-      <c r="E86" s="0">
-        <v>1</v>
-      </c>
-      <c r="F86" s="0"/>
+      <c r="E86" s="0"/>
+      <c r="F86" s="0">
+        <v>1</v>
+      </c>
       <c r="G86" s="0">
         <v>1000</v>
       </c>
@@ -5069,7 +5052,7 @@
       </c>
       <c r="V86" s="0"/>
       <c r="W86" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C86="","Missing blog title",""),IF(E86="","Missing slides per post",""),IF(OR(E86&lt;1,E86&gt;10),"Slides per post must be 1-10",""),IF(F86="","Missing URL",""),IF(G86="","Missing width",""),IF(H86="","Missing height",""),IF(I86="","Missing theme",""),IF(M86="","Missing hero type",""),IF(N86="","Missing image direction",""),IF(U86="","Missing status",""),IF(AND(J86="Custom",K86=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C86="","Missing blog title",""),IF(E86="","Missing URL",""),IF(F86="","Missing number of slides",""),IF(OR(F86&lt;1,F86&gt;10),"Number of slides must be 1-10",""),IF(G86="","Missing width",""),IF(H86="","Missing height",""),IF(I86="","Missing theme",""),IF(M86="","Missing hero type",""),IF(N86="","Missing image direction",""),IF(U86="","Missing status",""),IF(AND(J86="Custom",K86=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="87">
@@ -5079,10 +5062,10 @@
       <c r="B87" s="0"/>
       <c r="C87" s="0"/>
       <c r="D87" s="0"/>
-      <c r="E87" s="0">
-        <v>1</v>
-      </c>
-      <c r="F87" s="0"/>
+      <c r="E87" s="0"/>
+      <c r="F87" s="0">
+        <v>1</v>
+      </c>
       <c r="G87" s="0">
         <v>1000</v>
       </c>
@@ -5124,7 +5107,7 @@
       </c>
       <c r="V87" s="0"/>
       <c r="W87" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C87="","Missing blog title",""),IF(E87="","Missing slides per post",""),IF(OR(E87&lt;1,E87&gt;10),"Slides per post must be 1-10",""),IF(F87="","Missing URL",""),IF(G87="","Missing width",""),IF(H87="","Missing height",""),IF(I87="","Missing theme",""),IF(M87="","Missing hero type",""),IF(N87="","Missing image direction",""),IF(U87="","Missing status",""),IF(AND(J87="Custom",K87=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C87="","Missing blog title",""),IF(E87="","Missing URL",""),IF(F87="","Missing number of slides",""),IF(OR(F87&lt;1,F87&gt;10),"Number of slides must be 1-10",""),IF(G87="","Missing width",""),IF(H87="","Missing height",""),IF(I87="","Missing theme",""),IF(M87="","Missing hero type",""),IF(N87="","Missing image direction",""),IF(U87="","Missing status",""),IF(AND(J87="Custom",K87=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="88">
@@ -5134,10 +5117,10 @@
       <c r="B88" s="0"/>
       <c r="C88" s="0"/>
       <c r="D88" s="0"/>
-      <c r="E88" s="0">
-        <v>1</v>
-      </c>
-      <c r="F88" s="0"/>
+      <c r="E88" s="0"/>
+      <c r="F88" s="0">
+        <v>1</v>
+      </c>
       <c r="G88" s="0">
         <v>1000</v>
       </c>
@@ -5179,7 +5162,7 @@
       </c>
       <c r="V88" s="0"/>
       <c r="W88" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C88="","Missing blog title",""),IF(E88="","Missing slides per post",""),IF(OR(E88&lt;1,E88&gt;10),"Slides per post must be 1-10",""),IF(F88="","Missing URL",""),IF(G88="","Missing width",""),IF(H88="","Missing height",""),IF(I88="","Missing theme",""),IF(M88="","Missing hero type",""),IF(N88="","Missing image direction",""),IF(U88="","Missing status",""),IF(AND(J88="Custom",K88=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C88="","Missing blog title",""),IF(E88="","Missing URL",""),IF(F88="","Missing number of slides",""),IF(OR(F88&lt;1,F88&gt;10),"Number of slides must be 1-10",""),IF(G88="","Missing width",""),IF(H88="","Missing height",""),IF(I88="","Missing theme",""),IF(M88="","Missing hero type",""),IF(N88="","Missing image direction",""),IF(U88="","Missing status",""),IF(AND(J88="Custom",K88=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="89">
@@ -5189,10 +5172,10 @@
       <c r="B89" s="0"/>
       <c r="C89" s="0"/>
       <c r="D89" s="0"/>
-      <c r="E89" s="0">
-        <v>1</v>
-      </c>
-      <c r="F89" s="0"/>
+      <c r="E89" s="0"/>
+      <c r="F89" s="0">
+        <v>1</v>
+      </c>
       <c r="G89" s="0">
         <v>1000</v>
       </c>
@@ -5234,7 +5217,7 @@
       </c>
       <c r="V89" s="0"/>
       <c r="W89" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C89="","Missing blog title",""),IF(E89="","Missing slides per post",""),IF(OR(E89&lt;1,E89&gt;10),"Slides per post must be 1-10",""),IF(F89="","Missing URL",""),IF(G89="","Missing width",""),IF(H89="","Missing height",""),IF(I89="","Missing theme",""),IF(M89="","Missing hero type",""),IF(N89="","Missing image direction",""),IF(U89="","Missing status",""),IF(AND(J89="Custom",K89=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C89="","Missing blog title",""),IF(E89="","Missing URL",""),IF(F89="","Missing number of slides",""),IF(OR(F89&lt;1,F89&gt;10),"Number of slides must be 1-10",""),IF(G89="","Missing width",""),IF(H89="","Missing height",""),IF(I89="","Missing theme",""),IF(M89="","Missing hero type",""),IF(N89="","Missing image direction",""),IF(U89="","Missing status",""),IF(AND(J89="Custom",K89=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="90">
@@ -5244,10 +5227,10 @@
       <c r="B90" s="0"/>
       <c r="C90" s="0"/>
       <c r="D90" s="0"/>
-      <c r="E90" s="0">
-        <v>1</v>
-      </c>
-      <c r="F90" s="0"/>
+      <c r="E90" s="0"/>
+      <c r="F90" s="0">
+        <v>1</v>
+      </c>
       <c r="G90" s="0">
         <v>1000</v>
       </c>
@@ -5289,7 +5272,7 @@
       </c>
       <c r="V90" s="0"/>
       <c r="W90" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C90="","Missing blog title",""),IF(E90="","Missing slides per post",""),IF(OR(E90&lt;1,E90&gt;10),"Slides per post must be 1-10",""),IF(F90="","Missing URL",""),IF(G90="","Missing width",""),IF(H90="","Missing height",""),IF(I90="","Missing theme",""),IF(M90="","Missing hero type",""),IF(N90="","Missing image direction",""),IF(U90="","Missing status",""),IF(AND(J90="Custom",K90=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C90="","Missing blog title",""),IF(E90="","Missing URL",""),IF(F90="","Missing number of slides",""),IF(OR(F90&lt;1,F90&gt;10),"Number of slides must be 1-10",""),IF(G90="","Missing width",""),IF(H90="","Missing height",""),IF(I90="","Missing theme",""),IF(M90="","Missing hero type",""),IF(N90="","Missing image direction",""),IF(U90="","Missing status",""),IF(AND(J90="Custom",K90=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="91">
@@ -5299,10 +5282,10 @@
       <c r="B91" s="0"/>
       <c r="C91" s="0"/>
       <c r="D91" s="0"/>
-      <c r="E91" s="0">
-        <v>1</v>
-      </c>
-      <c r="F91" s="0"/>
+      <c r="E91" s="0"/>
+      <c r="F91" s="0">
+        <v>1</v>
+      </c>
       <c r="G91" s="0">
         <v>1000</v>
       </c>
@@ -5344,7 +5327,7 @@
       </c>
       <c r="V91" s="0"/>
       <c r="W91" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C91="","Missing blog title",""),IF(E91="","Missing slides per post",""),IF(OR(E91&lt;1,E91&gt;10),"Slides per post must be 1-10",""),IF(F91="","Missing URL",""),IF(G91="","Missing width",""),IF(H91="","Missing height",""),IF(I91="","Missing theme",""),IF(M91="","Missing hero type",""),IF(N91="","Missing image direction",""),IF(U91="","Missing status",""),IF(AND(J91="Custom",K91=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C91="","Missing blog title",""),IF(E91="","Missing URL",""),IF(F91="","Missing number of slides",""),IF(OR(F91&lt;1,F91&gt;10),"Number of slides must be 1-10",""),IF(G91="","Missing width",""),IF(H91="","Missing height",""),IF(I91="","Missing theme",""),IF(M91="","Missing hero type",""),IF(N91="","Missing image direction",""),IF(U91="","Missing status",""),IF(AND(J91="Custom",K91=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="92">
@@ -5354,10 +5337,10 @@
       <c r="B92" s="0"/>
       <c r="C92" s="0"/>
       <c r="D92" s="0"/>
-      <c r="E92" s="0">
-        <v>1</v>
-      </c>
-      <c r="F92" s="0"/>
+      <c r="E92" s="0"/>
+      <c r="F92" s="0">
+        <v>1</v>
+      </c>
       <c r="G92" s="0">
         <v>1000</v>
       </c>
@@ -5399,7 +5382,7 @@
       </c>
       <c r="V92" s="0"/>
       <c r="W92" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C92="","Missing blog title",""),IF(E92="","Missing slides per post",""),IF(OR(E92&lt;1,E92&gt;10),"Slides per post must be 1-10",""),IF(F92="","Missing URL",""),IF(G92="","Missing width",""),IF(H92="","Missing height",""),IF(I92="","Missing theme",""),IF(M92="","Missing hero type",""),IF(N92="","Missing image direction",""),IF(U92="","Missing status",""),IF(AND(J92="Custom",K92=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C92="","Missing blog title",""),IF(E92="","Missing URL",""),IF(F92="","Missing number of slides",""),IF(OR(F92&lt;1,F92&gt;10),"Number of slides must be 1-10",""),IF(G92="","Missing width",""),IF(H92="","Missing height",""),IF(I92="","Missing theme",""),IF(M92="","Missing hero type",""),IF(N92="","Missing image direction",""),IF(U92="","Missing status",""),IF(AND(J92="Custom",K92=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="93">
@@ -5409,10 +5392,10 @@
       <c r="B93" s="0"/>
       <c r="C93" s="0"/>
       <c r="D93" s="0"/>
-      <c r="E93" s="0">
-        <v>1</v>
-      </c>
-      <c r="F93" s="0"/>
+      <c r="E93" s="0"/>
+      <c r="F93" s="0">
+        <v>1</v>
+      </c>
       <c r="G93" s="0">
         <v>1000</v>
       </c>
@@ -5454,7 +5437,7 @@
       </c>
       <c r="V93" s="0"/>
       <c r="W93" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C93="","Missing blog title",""),IF(E93="","Missing slides per post",""),IF(OR(E93&lt;1,E93&gt;10),"Slides per post must be 1-10",""),IF(F93="","Missing URL",""),IF(G93="","Missing width",""),IF(H93="","Missing height",""),IF(I93="","Missing theme",""),IF(M93="","Missing hero type",""),IF(N93="","Missing image direction",""),IF(U93="","Missing status",""),IF(AND(J93="Custom",K93=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C93="","Missing blog title",""),IF(E93="","Missing URL",""),IF(F93="","Missing number of slides",""),IF(OR(F93&lt;1,F93&gt;10),"Number of slides must be 1-10",""),IF(G93="","Missing width",""),IF(H93="","Missing height",""),IF(I93="","Missing theme",""),IF(M93="","Missing hero type",""),IF(N93="","Missing image direction",""),IF(U93="","Missing status",""),IF(AND(J93="Custom",K93=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="94">
@@ -5464,10 +5447,10 @@
       <c r="B94" s="0"/>
       <c r="C94" s="0"/>
       <c r="D94" s="0"/>
-      <c r="E94" s="0">
-        <v>1</v>
-      </c>
-      <c r="F94" s="0"/>
+      <c r="E94" s="0"/>
+      <c r="F94" s="0">
+        <v>1</v>
+      </c>
       <c r="G94" s="0">
         <v>1000</v>
       </c>
@@ -5509,7 +5492,7 @@
       </c>
       <c r="V94" s="0"/>
       <c r="W94" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C94="","Missing blog title",""),IF(E94="","Missing slides per post",""),IF(OR(E94&lt;1,E94&gt;10),"Slides per post must be 1-10",""),IF(F94="","Missing URL",""),IF(G94="","Missing width",""),IF(H94="","Missing height",""),IF(I94="","Missing theme",""),IF(M94="","Missing hero type",""),IF(N94="","Missing image direction",""),IF(U94="","Missing status",""),IF(AND(J94="Custom",K94=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C94="","Missing blog title",""),IF(E94="","Missing URL",""),IF(F94="","Missing number of slides",""),IF(OR(F94&lt;1,F94&gt;10),"Number of slides must be 1-10",""),IF(G94="","Missing width",""),IF(H94="","Missing height",""),IF(I94="","Missing theme",""),IF(M94="","Missing hero type",""),IF(N94="","Missing image direction",""),IF(U94="","Missing status",""),IF(AND(J94="Custom",K94=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="95">
@@ -5519,10 +5502,10 @@
       <c r="B95" s="0"/>
       <c r="C95" s="0"/>
       <c r="D95" s="0"/>
-      <c r="E95" s="0">
-        <v>1</v>
-      </c>
-      <c r="F95" s="0"/>
+      <c r="E95" s="0"/>
+      <c r="F95" s="0">
+        <v>1</v>
+      </c>
       <c r="G95" s="0">
         <v>1000</v>
       </c>
@@ -5564,7 +5547,7 @@
       </c>
       <c r="V95" s="0"/>
       <c r="W95" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C95="","Missing blog title",""),IF(E95="","Missing slides per post",""),IF(OR(E95&lt;1,E95&gt;10),"Slides per post must be 1-10",""),IF(F95="","Missing URL",""),IF(G95="","Missing width",""),IF(H95="","Missing height",""),IF(I95="","Missing theme",""),IF(M95="","Missing hero type",""),IF(N95="","Missing image direction",""),IF(U95="","Missing status",""),IF(AND(J95="Custom",K95=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C95="","Missing blog title",""),IF(E95="","Missing URL",""),IF(F95="","Missing number of slides",""),IF(OR(F95&lt;1,F95&gt;10),"Number of slides must be 1-10",""),IF(G95="","Missing width",""),IF(H95="","Missing height",""),IF(I95="","Missing theme",""),IF(M95="","Missing hero type",""),IF(N95="","Missing image direction",""),IF(U95="","Missing status",""),IF(AND(J95="Custom",K95=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="96">
@@ -5574,10 +5557,10 @@
       <c r="B96" s="0"/>
       <c r="C96" s="0"/>
       <c r="D96" s="0"/>
-      <c r="E96" s="0">
-        <v>1</v>
-      </c>
-      <c r="F96" s="0"/>
+      <c r="E96" s="0"/>
+      <c r="F96" s="0">
+        <v>1</v>
+      </c>
       <c r="G96" s="0">
         <v>1000</v>
       </c>
@@ -5619,7 +5602,7 @@
       </c>
       <c r="V96" s="0"/>
       <c r="W96" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C96="","Missing blog title",""),IF(E96="","Missing slides per post",""),IF(OR(E96&lt;1,E96&gt;10),"Slides per post must be 1-10",""),IF(F96="","Missing URL",""),IF(G96="","Missing width",""),IF(H96="","Missing height",""),IF(I96="","Missing theme",""),IF(M96="","Missing hero type",""),IF(N96="","Missing image direction",""),IF(U96="","Missing status",""),IF(AND(J96="Custom",K96=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C96="","Missing blog title",""),IF(E96="","Missing URL",""),IF(F96="","Missing number of slides",""),IF(OR(F96&lt;1,F96&gt;10),"Number of slides must be 1-10",""),IF(G96="","Missing width",""),IF(H96="","Missing height",""),IF(I96="","Missing theme",""),IF(M96="","Missing hero type",""),IF(N96="","Missing image direction",""),IF(U96="","Missing status",""),IF(AND(J96="Custom",K96=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="97">
@@ -5629,10 +5612,10 @@
       <c r="B97" s="0"/>
       <c r="C97" s="0"/>
       <c r="D97" s="0"/>
-      <c r="E97" s="0">
-        <v>1</v>
-      </c>
-      <c r="F97" s="0"/>
+      <c r="E97" s="0"/>
+      <c r="F97" s="0">
+        <v>1</v>
+      </c>
       <c r="G97" s="0">
         <v>1000</v>
       </c>
@@ -5674,7 +5657,7 @@
       </c>
       <c r="V97" s="0"/>
       <c r="W97" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C97="","Missing blog title",""),IF(E97="","Missing slides per post",""),IF(OR(E97&lt;1,E97&gt;10),"Slides per post must be 1-10",""),IF(F97="","Missing URL",""),IF(G97="","Missing width",""),IF(H97="","Missing height",""),IF(I97="","Missing theme",""),IF(M97="","Missing hero type",""),IF(N97="","Missing image direction",""),IF(U97="","Missing status",""),IF(AND(J97="Custom",K97=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C97="","Missing blog title",""),IF(E97="","Missing URL",""),IF(F97="","Missing number of slides",""),IF(OR(F97&lt;1,F97&gt;10),"Number of slides must be 1-10",""),IF(G97="","Missing width",""),IF(H97="","Missing height",""),IF(I97="","Missing theme",""),IF(M97="","Missing hero type",""),IF(N97="","Missing image direction",""),IF(U97="","Missing status",""),IF(AND(J97="Custom",K97=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="98">
@@ -5684,10 +5667,10 @@
       <c r="B98" s="0"/>
       <c r="C98" s="0"/>
       <c r="D98" s="0"/>
-      <c r="E98" s="0">
-        <v>1</v>
-      </c>
-      <c r="F98" s="0"/>
+      <c r="E98" s="0"/>
+      <c r="F98" s="0">
+        <v>1</v>
+      </c>
       <c r="G98" s="0">
         <v>1000</v>
       </c>
@@ -5729,7 +5712,7 @@
       </c>
       <c r="V98" s="0"/>
       <c r="W98" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C98="","Missing blog title",""),IF(E98="","Missing slides per post",""),IF(OR(E98&lt;1,E98&gt;10),"Slides per post must be 1-10",""),IF(F98="","Missing URL",""),IF(G98="","Missing width",""),IF(H98="","Missing height",""),IF(I98="","Missing theme",""),IF(M98="","Missing hero type",""),IF(N98="","Missing image direction",""),IF(U98="","Missing status",""),IF(AND(J98="Custom",K98=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C98="","Missing blog title",""),IF(E98="","Missing URL",""),IF(F98="","Missing number of slides",""),IF(OR(F98&lt;1,F98&gt;10),"Number of slides must be 1-10",""),IF(G98="","Missing width",""),IF(H98="","Missing height",""),IF(I98="","Missing theme",""),IF(M98="","Missing hero type",""),IF(N98="","Missing image direction",""),IF(U98="","Missing status",""),IF(AND(J98="Custom",K98=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="99">
@@ -5739,10 +5722,10 @@
       <c r="B99" s="0"/>
       <c r="C99" s="0"/>
       <c r="D99" s="0"/>
-      <c r="E99" s="0">
-        <v>1</v>
-      </c>
-      <c r="F99" s="0"/>
+      <c r="E99" s="0"/>
+      <c r="F99" s="0">
+        <v>1</v>
+      </c>
       <c r="G99" s="0">
         <v>1000</v>
       </c>
@@ -5784,7 +5767,7 @@
       </c>
       <c r="V99" s="0"/>
       <c r="W99" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C99="","Missing blog title",""),IF(E99="","Missing slides per post",""),IF(OR(E99&lt;1,E99&gt;10),"Slides per post must be 1-10",""),IF(F99="","Missing URL",""),IF(G99="","Missing width",""),IF(H99="","Missing height",""),IF(I99="","Missing theme",""),IF(M99="","Missing hero type",""),IF(N99="","Missing image direction",""),IF(U99="","Missing status",""),IF(AND(J99="Custom",K99=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C99="","Missing blog title",""),IF(E99="","Missing URL",""),IF(F99="","Missing number of slides",""),IF(OR(F99&lt;1,F99&gt;10),"Number of slides must be 1-10",""),IF(G99="","Missing width",""),IF(H99="","Missing height",""),IF(I99="","Missing theme",""),IF(M99="","Missing hero type",""),IF(N99="","Missing image direction",""),IF(U99="","Missing status",""),IF(AND(J99="Custom",K99=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="100">
@@ -5794,10 +5777,10 @@
       <c r="B100" s="0"/>
       <c r="C100" s="0"/>
       <c r="D100" s="0"/>
-      <c r="E100" s="0">
-        <v>1</v>
-      </c>
-      <c r="F100" s="0"/>
+      <c r="E100" s="0"/>
+      <c r="F100" s="0">
+        <v>1</v>
+      </c>
       <c r="G100" s="0">
         <v>1000</v>
       </c>
@@ -5839,7 +5822,7 @@
       </c>
       <c r="V100" s="0"/>
       <c r="W100" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C100="","Missing blog title",""),IF(E100="","Missing slides per post",""),IF(OR(E100&lt;1,E100&gt;10),"Slides per post must be 1-10",""),IF(F100="","Missing URL",""),IF(G100="","Missing width",""),IF(H100="","Missing height",""),IF(I100="","Missing theme",""),IF(M100="","Missing hero type",""),IF(N100="","Missing image direction",""),IF(U100="","Missing status",""),IF(AND(J100="Custom",K100=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C100="","Missing blog title",""),IF(E100="","Missing URL",""),IF(F100="","Missing number of slides",""),IF(OR(F100&lt;1,F100&gt;10),"Number of slides must be 1-10",""),IF(G100="","Missing width",""),IF(H100="","Missing height",""),IF(I100="","Missing theme",""),IF(M100="","Missing hero type",""),IF(N100="","Missing image direction",""),IF(U100="","Missing status",""),IF(AND(J100="Custom",K100=""),"Custom visible text missing",""))</f>
       </c>
     </row>
     <row r="101">
@@ -5849,10 +5832,10 @@
       <c r="B101" s="0"/>
       <c r="C101" s="0"/>
       <c r="D101" s="0"/>
-      <c r="E101" s="0">
-        <v>1</v>
-      </c>
-      <c r="F101" s="0"/>
+      <c r="E101" s="0"/>
+      <c r="F101" s="0">
+        <v>1</v>
+      </c>
       <c r="G101" s="0">
         <v>1000</v>
       </c>
@@ -5894,16 +5877,16 @@
       </c>
       <c r="V101" s="0"/>
       <c r="W101" s="0">
-        <f>TEXTJOIN("; ",TRUE,IF(C101="","Missing blog title",""),IF(E101="","Missing slides per post",""),IF(OR(E101&lt;1,E101&gt;10),"Slides per post must be 1-10",""),IF(F101="","Missing URL",""),IF(G101="","Missing width",""),IF(H101="","Missing height",""),IF(I101="","Missing theme",""),IF(M101="","Missing hero type",""),IF(N101="","Missing image direction",""),IF(U101="","Missing status",""),IF(AND(J101="Custom",K101=""),"Custom visible text missing",""))</f>
+        <f>TEXTJOIN("; ",TRUE,IF(C101="","Missing blog title",""),IF(E101="","Missing URL",""),IF(F101="","Missing number of slides",""),IF(OR(F101&lt;1,F101&gt;10),"Number of slides must be 1-10",""),IF(G101="","Missing width",""),IF(H101="","Missing height",""),IF(I101="","Missing theme",""),IF(M101="","Missing hero type",""),IF(N101="","Missing image direction",""),IF(U101="","Missing status",""),IF(AND(J101="Custom",K101=""),"Custom visible text missing",""))</f>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:W101"/>
   <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="E2:E101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="F2:F101">
       <formula1>Lists!$H$2:$H$11</formula1>
       <promptTitle>Choose a value</promptTitle>
-      <prompt>Choose slides per post: 1 for a single image, 2-10 for carousel slides.</prompt>
+      <prompt>Choose number of slides. Defaults to 1.</prompt>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="I2:I101">
       <formula1>Lists!$A$2:$A$4</formula1>
@@ -5950,9 +5933,8 @@
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="52" customWidth="1"/>
-    <col min="7" max="23" width="24" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
+    <col min="6" max="23" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5978,12 +5960,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Slides per post</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>Number of slides</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -6093,13 +6075,13 @@
           <t>Cars24 announces Labs, a $20M AI bet to build, partner with, and invest in AI-native companies.</t>
         </is>
       </c>
-      <c r="E2" s="0">
-        <v>1</v>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/introducing-cars24-labs-cars24s-20-million-bet-on-ai</t>
         </is>
+      </c>
+      <c r="F2" s="0">
+        <v>1</v>
       </c>
       <c r="G2" s="0">
         <v>1000</v>
@@ -6188,13 +6170,13 @@
           <t>Explains why broken RC transfer systems create legal risk and why Cars24 is pushing for reform.</t>
         </is>
       </c>
-      <c r="E3" s="0">
-        <v>1</v>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/rc-transfer-the-broken-system-we-are-fixing-for-india</t>
         </is>
+      </c>
+      <c r="F3" s="0">
+        <v>1</v>
       </c>
       <c r="G3" s="0">
         <v>1000</v>
@@ -6283,13 +6265,13 @@
           <t>Breaks down Cars24's first fully automated AI loan reference-check workflow with no human intervention.</t>
         </is>
       </c>
-      <c r="E4" s="0">
-        <v>1</v>
-      </c>
-      <c r="F4" s="0" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/no-human-in-the-loop-cars24-first-ai-loan-workflow</t>
         </is>
+      </c>
+      <c r="F4" s="0">
+        <v>1</v>
       </c>
       <c r="G4" s="0">
         <v>1000</v>
@@ -6378,13 +6360,13 @@
           <t>A reflection on the blind spots companies develop as they grow and how teams can keep clarity intact.</t>
         </is>
       </c>
-      <c r="E5" s="0">
-        <v>1</v>
-      </c>
-      <c r="F5" s="0" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/what-orgs-stop-seeing-as-they-scale</t>
         </is>
+      </c>
+      <c r="F5" s="0">
+        <v>1</v>
       </c>
       <c r="G5" s="0">
         <v>1000</v>
@@ -6473,13 +6455,13 @@
           <t>Outlines the values and operating principles Cars24 wants to carry into its next phase of growth.</t>
         </is>
       </c>
-      <c r="E6" s="0">
-        <v>1</v>
-      </c>
-      <c r="F6" s="0" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/the-values-for-next-chapter-of-cars24</t>
         </is>
+      </c>
+      <c r="F6" s="0">
+        <v>1</v>
       </c>
       <c r="G6" s="0">
         <v>1000</v>
@@ -6568,13 +6550,13 @@
           <t>Shows how long-term brand thinking and strategic bets helped growth rise despite lower marketing spend.</t>
         </is>
       </c>
-      <c r="E7" s="0">
-        <v>1</v>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/long-term-thinking-in-marketing-pays-off</t>
         </is>
+      </c>
+      <c r="F7" s="0">
+        <v>1</v>
       </c>
       <c r="G7" s="0">
         <v>1000</v>
@@ -6663,13 +6645,13 @@
           <t>Shares the launch and early success of Cars24's all-women auto hub in Saket, Delhi NCR.</t>
         </is>
       </c>
-      <c r="E8" s="0">
-        <v>1</v>
-      </c>
-      <c r="F8" s="0" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/all-women-cars24-auto-hub-in-delhi-ncr</t>
         </is>
+      </c>
+      <c r="F8" s="0">
+        <v>1</v>
       </c>
       <c r="G8" s="0">
         <v>1000</v>
@@ -6758,13 +6740,13 @@
           <t>Explains how Cars24 rebuilt its used-car pricing system using data science, modelling, and feedback loops.</t>
         </is>
       </c>
-      <c r="E9" s="0">
-        <v>1</v>
-      </c>
-      <c r="F9" s="0" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/how-cars24-prices-your-pre-owned-car</t>
         </is>
+      </c>
+      <c r="F9" s="0">
+        <v>1</v>
       </c>
       <c r="G9" s="0">
         <v>1000</v>
@@ -6853,13 +6835,13 @@
           <t>A people-focused story about the frontline teams and leaders shaping customer trust at Cars24.</t>
         </is>
       </c>
-      <c r="E10" s="0">
-        <v>1</v>
-      </c>
-      <c r="F10" s="0" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/the-three-at-the-front</t>
         </is>
+      </c>
+      <c r="F10" s="0">
+        <v>1</v>
       </c>
       <c r="G10" s="0">
         <v>1000</v>
@@ -6948,13 +6930,13 @@
           <t>Tells how an Autonaut used AI and Cloudflare to build an internal tool now used by 1000+ people.</t>
         </is>
       </c>
-      <c r="E11" s="0">
-        <v>1</v>
-      </c>
-      <c r="F11" s="0" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/how-a-non-engineer-built-the-tool-1000-people-at-cars24-now-use</t>
         </is>
+      </c>
+      <c r="F11" s="0">
+        <v>1</v>
       </c>
       <c r="G11" s="0">
         <v>1000</v>
@@ -7043,13 +7025,13 @@
           <t>Argues that analytics teams should influence business choices, not just report what already happened.</t>
         </is>
       </c>
-      <c r="E12" s="0">
-        <v>1</v>
-      </c>
-      <c r="F12" s="0" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/analytics-drive-decisions</t>
         </is>
+      </c>
+      <c r="F12" s="0">
+        <v>1</v>
       </c>
       <c r="G12" s="0">
         <v>1000</v>
@@ -7138,13 +7120,13 @@
           <t>Announces Gajendra Jangid stepping back from his co-founder role while continuing to contribute to Cars24's mission.</t>
         </is>
       </c>
-      <c r="E13" s="0">
-        <v>1</v>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/gajendra-jangid-steps-down-from-co-founder</t>
         </is>
+      </c>
+      <c r="F13" s="0">
+        <v>1</v>
       </c>
       <c r="G13" s="0">
         <v>1000</v>
@@ -7233,13 +7215,13 @@
           <t>Frames Cars24's AI-era culture around one core identity: people who build, solve, and own outcomes.</t>
         </is>
       </c>
-      <c r="E14" s="0">
-        <v>1</v>
-      </c>
-      <c r="F14" s="0" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/only-role-in-the-company-builder</t>
         </is>
+      </c>
+      <c r="F14" s="0">
+        <v>1</v>
       </c>
       <c r="G14" s="0">
         <v>1000</v>
@@ -7328,13 +7310,13 @@
           <t>Explains how RC transfer gaps affect sellers, buyers, and the broader used-car ecosystem in India.</t>
         </is>
       </c>
-      <c r="E15" s="0">
-        <v>1</v>
-      </c>
-      <c r="F15" s="0" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/rc-crisis-in-india</t>
         </is>
+      </c>
+      <c r="F15" s="0">
+        <v>1</v>
       </c>
       <c r="G15" s="0">
         <v>1000</v>
@@ -7423,13 +7405,13 @@
           <t>Reviews Cars24's first year of AI transformation and the move toward an AI-first customer experience.</t>
         </is>
       </c>
-      <c r="E16" s="0">
-        <v>1</v>
-      </c>
-      <c r="F16" s="0" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/one-year-into-our-ai-journey-cars24</t>
         </is>
+      </c>
+      <c r="F16" s="0">
+        <v>1</v>
       </c>
       <c r="G16" s="0">
         <v>1000</v>
@@ -7518,13 +7500,13 @@
           <t>Covers the redesign of Cars24 showrooms and the role of people, service, and experience in that transformation.</t>
         </is>
       </c>
-      <c r="E17" s="0">
-        <v>1</v>
-      </c>
-      <c r="F17" s="0" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/showroom-transformation-at-cars24</t>
         </is>
+      </c>
+      <c r="F17" s="0">
+        <v>1</v>
       </c>
       <c r="G17" s="0">
         <v>1000</v>
@@ -7613,13 +7595,13 @@
           <t>A reflective piece on persistence, effort, and how progress compounds even when results are not immediate.</t>
         </is>
       </c>
-      <c r="E18" s="0">
-        <v>1</v>
-      </c>
-      <c r="F18" s="0" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/the-sisyphus-story-by-utkarsh</t>
         </is>
+      </c>
+      <c r="F18" s="0">
+        <v>1</v>
       </c>
       <c r="G18" s="0">
         <v>1000</v>
@@ -7708,13 +7690,13 @@
           <t>A personal Autonaut story about growth, learning, and career experience inside Cars24.</t>
         </is>
       </c>
-      <c r="E19" s="0">
-        <v>1</v>
-      </c>
-      <c r="F19" s="0" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/jerusa-dimka-cars24-journey</t>
         </is>
+      </c>
+      <c r="F19" s="0">
+        <v>1</v>
       </c>
       <c r="G19" s="0">
         <v>1000</v>
@@ -7803,13 +7785,13 @@
           <t>Explains how repainting can affect resale value, buyer perception, and trust in a used car.</t>
         </is>
       </c>
-      <c r="E20" s="0">
-        <v>1</v>
-      </c>
-      <c r="F20" s="0" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/repainting-a-used-car-does-it-affect-resale-value-safety-or-performance</t>
         </is>
+      </c>
+      <c r="F20" s="0">
+        <v>1</v>
       </c>
       <c r="G20" s="0">
         <v>1000</v>
@@ -7898,13 +7880,13 @@
           <t>Celebrates the people behind Cars24's customer and operational experience.</t>
         </is>
       </c>
-      <c r="E21" s="0">
-        <v>1</v>
-      </c>
-      <c r="F21" s="0" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/people-behind-the-drive</t>
         </is>
+      </c>
+      <c r="F21" s="0">
+        <v>1</v>
       </c>
       <c r="G21" s="0">
         <v>1000</v>
@@ -7993,13 +7975,13 @@
           <t>Introduces Cars24's lifetime warranty promise covering key mechanical components for eligible cars.</t>
         </is>
       </c>
-      <c r="E22" s="0">
-        <v>1</v>
-      </c>
-      <c r="F22" s="0" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/first-lifetime-warranty</t>
         </is>
+      </c>
+      <c r="F22" s="0">
+        <v>1</v>
       </c>
       <c r="G22" s="0">
         <v>1000</v>
@@ -8088,13 +8070,13 @@
           <t>A culture story about personal growth, support, and finding momentum at Cars24.</t>
         </is>
       </c>
-      <c r="E23" s="0">
-        <v>1</v>
-      </c>
-      <c r="F23" s="0" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/from-cocoon-to-career</t>
         </is>
+      </c>
+      <c r="F23" s="0">
+        <v>1</v>
       </c>
       <c r="G23" s="0">
         <v>1000</v>
@@ -8183,13 +8165,13 @@
           <t>Reflects on humility, learning, and team-first decision-making as a path to winning.</t>
         </is>
       </c>
-      <c r="E24" s="0">
-        <v>1</v>
-      </c>
-      <c r="F24" s="0" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/winning-isnt-about-being-right</t>
         </is>
+      </c>
+      <c r="F24" s="0">
+        <v>1</v>
       </c>
       <c r="G24" s="0">
         <v>1000</v>
@@ -8278,13 +8260,13 @@
           <t>Connects Cars24's work to the broader human desire to move forward and build better systems.</t>
         </is>
       </c>
-      <c r="E25" s="0">
-        <v>1</v>
-      </c>
-      <c r="F25" s="0" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/on-evolution</t>
         </is>
+      </c>
+      <c r="F25" s="0">
+        <v>1</v>
       </c>
       <c r="G25" s="0">
         <v>1000</v>
@@ -8373,13 +8355,13 @@
           <t>Explains why early ownership support matters for buyer confidence, trust, and long-term satisfaction.</t>
         </is>
       </c>
-      <c r="E26" s="0">
-        <v>1</v>
-      </c>
-      <c r="F26" s="0" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/why-first-30-days-matter-after-buying-used-car</t>
         </is>
+      </c>
+      <c r="F26" s="0">
+        <v>1</v>
       </c>
       <c r="G26" s="0">
         <v>1000</v>
@@ -8468,13 +8450,13 @@
           <t>Shares engineering lessons from building reliable Node.js backend-for-frontend systems at scale.</t>
         </is>
       </c>
-      <c r="E27" s="0">
-        <v>1</v>
-      </c>
-      <c r="F27" s="0" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/building-resilient-node-js</t>
         </is>
+      </c>
+      <c r="F27" s="0">
+        <v>1</v>
       </c>
       <c r="G27" s="0">
         <v>1000</v>
@@ -8563,13 +8545,13 @@
           <t>Explains common customer misunderstandings during car selling and how better clarity can improve trust.</t>
         </is>
       </c>
-      <c r="E28" s="0">
-        <v>1</v>
-      </c>
-      <c r="F28" s="0" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/car-selling-process</t>
         </is>
+      </c>
+      <c r="F28" s="0">
+        <v>1</v>
       </c>
       <c r="G28" s="0">
         <v>1000</v>
@@ -8658,13 +8640,13 @@
           <t>Looks at Voice AI reliability, hallucination risks, and safeguards needed for real-world use.</t>
         </is>
       </c>
-      <c r="E29" s="0">
-        <v>1</v>
-      </c>
-      <c r="F29" s="0" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/when-voice-ai-loses-track-of-reality</t>
         </is>
+      </c>
+      <c r="F29" s="0">
+        <v>1</v>
       </c>
       <c r="G29" s="0">
         <v>1000</v>
@@ -8753,13 +8735,13 @@
           <t>Reflects on founder decision fatigue and the challenge of maintaining clarity under high decision load.</t>
         </is>
       </c>
-      <c r="E30" s="0">
-        <v>1</v>
-      </c>
-      <c r="F30" s="0" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/founders-fog</t>
         </is>
+      </c>
+      <c r="F30" s="0">
+        <v>1</v>
       </c>
       <c r="G30" s="0">
         <v>1000</v>
@@ -8848,13 +8830,13 @@
           <t>Explains Cars24's ESOP philosophy around employee trust, liquidity, and fair ownership terms.</t>
         </is>
       </c>
-      <c r="E31" s="0">
-        <v>1</v>
-      </c>
-      <c r="F31" s="0" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/cars24-esop-strategy</t>
         </is>
+      </c>
+      <c r="F31" s="0">
+        <v>1</v>
       </c>
       <c r="G31" s="0">
         <v>1000</v>
@@ -8943,13 +8925,13 @@
           <t>Reflects on Cars24 Arabia's growth, profitability milestone, and sharper purpose for the year ahead.</t>
         </is>
       </c>
-      <c r="E32" s="0">
-        <v>1</v>
-      </c>
-      <c r="F32" s="0" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/a-new-year-a-clearer-purpose</t>
         </is>
+      </c>
+      <c r="F32" s="0">
+        <v>1</v>
       </c>
       <c r="G32" s="0">
         <v>1000</v>
@@ -9038,13 +9020,13 @@
           <t>A reflection on hustle culture, ambition, and the personal trade-offs that come with constant motion.</t>
         </is>
       </c>
-      <c r="E33" s="0">
-        <v>1</v>
-      </c>
-      <c r="F33" s="0" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/constant-hustle</t>
         </is>
+      </c>
+      <c r="F33" s="0">
+        <v>1</v>
       </c>
       <c r="G33" s="0">
         <v>1000</v>
@@ -9133,13 +9115,13 @@
           <t>A practical first-aid and action guide for what drivers should do immediately after a road accident.</t>
         </is>
       </c>
-      <c r="E34" s="0">
-        <v>1</v>
-      </c>
-      <c r="F34" s="0" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/a-complete-first-aid-guide</t>
         </is>
+      </c>
+      <c r="F34" s="0">
+        <v>1</v>
       </c>
       <c r="G34" s="0">
         <v>1000</v>
@@ -9228,13 +9210,13 @@
           <t>Reflects on work culture, personal values, and how everyday habits shape the way teams operate.</t>
         </is>
       </c>
-      <c r="E35" s="0">
-        <v>1</v>
-      </c>
-      <c r="F35" s="0" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/how-we-work</t>
         </is>
+      </c>
+      <c r="F35" s="0">
+        <v>1</v>
       </c>
       <c r="G35" s="0">
         <v>1000</v>
@@ -9323,13 +9305,13 @@
           <t>Explains crash-claim compensation basics and what people should know after a road accident.</t>
         </is>
       </c>
-      <c r="E36" s="0">
-        <v>1</v>
-      </c>
-      <c r="F36" s="0" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/crash-claim-compensation-guide</t>
         </is>
+      </c>
+      <c r="F36" s="0">
+        <v>1</v>
       </c>
       <c r="G36" s="0">
         <v>1000</v>
@@ -9418,13 +9400,13 @@
           <t>Describes how feedback loops and observability can help teams turn signals into visible improvements.</t>
         </is>
       </c>
-      <c r="E37" s="0">
-        <v>1</v>
-      </c>
-      <c r="F37" s="0" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/from-feedback-to-visible-change</t>
         </is>
+      </c>
+      <c r="F37" s="0">
+        <v>1</v>
       </c>
       <c r="G37" s="0">
         <v>1000</v>
@@ -9513,13 +9495,13 @@
           <t>Makes the case that consistent execution on unglamorous fundamentals creates durable excellence.</t>
         </is>
       </c>
-      <c r="E38" s="0">
-        <v>1</v>
-      </c>
-      <c r="F38" s="0" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/mastering-the-boring</t>
         </is>
+      </c>
+      <c r="F38" s="0">
+        <v>1</v>
       </c>
       <c r="G38" s="0">
         <v>1000</v>
@@ -9608,13 +9590,13 @@
           <t>Explores how road hazards create serious safety risks and why the issue needs more attention.</t>
         </is>
       </c>
-      <c r="E39" s="0">
-        <v>1</v>
-      </c>
-      <c r="F39" s="0" t="inlineStr">
+      <c r="E39" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/when-lives-collide</t>
         </is>
+      </c>
+      <c r="F39" s="0">
+        <v>1</v>
       </c>
       <c r="G39" s="0">
         <v>1000</v>
@@ -9703,13 +9685,13 @@
           <t>Explains Bharat NCAP safety ratings and what car buyers should understand about crash-test stars.</t>
         </is>
       </c>
-      <c r="E40" s="0">
-        <v>1</v>
-      </c>
-      <c r="F40" s="0" t="inlineStr">
+      <c r="E40" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/decoding-bharat-ncap</t>
         </is>
+      </c>
+      <c r="F40" s="0">
+        <v>1</v>
       </c>
       <c r="G40" s="0">
         <v>1000</v>
@@ -9798,13 +9780,13 @@
           <t>A personal journey story about curiosity, growth, and learning as part of the Cars24 team.</t>
         </is>
       </c>
-      <c r="E41" s="0">
-        <v>1</v>
-      </c>
-      <c r="F41" s="0" t="inlineStr">
+      <c r="E41" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/journey-with-cars24-riya-jain</t>
         </is>
+      </c>
+      <c r="F41" s="0">
+        <v>1</v>
       </c>
       <c r="G41" s="0">
         <v>1000</v>
@@ -9893,13 +9875,13 @@
           <t>A technical walkthrough on using Cloudflare Workers to improve Gupshup campaign workflows.</t>
         </is>
       </c>
-      <c r="E42" s="0">
-        <v>1</v>
-      </c>
-      <c r="F42" s="0" t="inlineStr">
+      <c r="E42" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/supercharge-gupshup-campaigns</t>
         </is>
+      </c>
+      <c r="F42" s="0">
+        <v>1</v>
       </c>
       <c r="G42" s="0">
         <v>1000</v>
@@ -9988,13 +9970,13 @@
           <t>Introduces Cars24's Vehicle Health Report by Orbit and how it helps understand vehicle condition.</t>
         </is>
       </c>
-      <c r="E43" s="0">
-        <v>1</v>
-      </c>
-      <c r="F43" s="0" t="inlineStr">
+      <c r="E43" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/cars24-indias-vehicle-health-report-by-orbit</t>
         </is>
+      </c>
+      <c r="F43" s="0">
+        <v>1</v>
       </c>
       <c r="G43" s="0">
         <v>1000</v>
@@ -10083,13 +10065,13 @@
           <t>Explores how personalisation can improve discovery, trust, and conversion in automotive e-commerce.</t>
         </is>
       </c>
-      <c r="E44" s="0">
-        <v>1</v>
-      </c>
-      <c r="F44" s="0" t="inlineStr">
+      <c r="E44" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/power-of-personalisation</t>
         </is>
+      </c>
+      <c r="F44" s="0">
+        <v>1</v>
       </c>
       <c r="G44" s="0">
         <v>1000</v>
@@ -10178,13 +10160,13 @@
           <t>Highlights the people who bring calm, reliability, and execution strength during chaotic moments.</t>
         </is>
       </c>
-      <c r="E45" s="0">
-        <v>1</v>
-      </c>
-      <c r="F45" s="0" t="inlineStr">
+      <c r="E45" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/quiet-heroes</t>
         </is>
+      </c>
+      <c r="F45" s="0">
+        <v>1</v>
       </c>
       <c r="G45" s="0">
         <v>1000</v>
@@ -10273,13 +10255,13 @@
           <t>Shares lessons from building OCR systems for messy, real-world document processing at scale.</t>
         </is>
       </c>
-      <c r="E46" s="0">
-        <v>1</v>
-      </c>
-      <c r="F46" s="0" t="inlineStr">
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/cracking-ocr</t>
         </is>
+      </c>
+      <c r="F46" s="0">
+        <v>1</v>
       </c>
       <c r="G46" s="0">
         <v>1000</v>
@@ -10368,13 +10350,13 @@
           <t>Explains how Cars24 built real-time data streaming into dashboards and APIs for faster visibility.</t>
         </is>
       </c>
-      <c r="E47" s="0">
-        <v>1</v>
-      </c>
-      <c r="F47" s="0" t="inlineStr">
+      <c r="E47" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/real-time-all-the-time</t>
         </is>
+      </c>
+      <c r="F47" s="0">
+        <v>1</v>
       </c>
       <c r="G47" s="0">
         <v>1000</v>
@@ -10463,13 +10445,13 @@
           <t>Explains how Cars24 fine-tuned Whisper to improve call transcription and intelligence for auto-domain conversations.</t>
         </is>
       </c>
-      <c r="E48" s="0">
-        <v>1</v>
-      </c>
-      <c r="F48" s="0" t="inlineStr">
+      <c r="E48" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/cars24-call-intelligence</t>
         </is>
+      </c>
+      <c r="F48" s="0">
+        <v>1</v>
       </c>
       <c r="G48" s="0">
         <v>1000</v>
@@ -10558,13 +10540,13 @@
           <t>A personal reflection on two years of learning, growth, and contribution at Cars24.</t>
         </is>
       </c>
-      <c r="E49" s="0">
-        <v>1</v>
-      </c>
-      <c r="F49" s="0" t="inlineStr">
+      <c r="E49" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/my-journey-with-cars24-swena</t>
         </is>
+      </c>
+      <c r="F49" s="0">
+        <v>1</v>
       </c>
       <c r="G49" s="0">
         <v>1000</v>
@@ -10653,13 +10635,13 @@
           <t>Explores how Rive can help create interactive motion and richer product experiences.</t>
         </is>
       </c>
-      <c r="E50" s="0">
-        <v>1</v>
-      </c>
-      <c r="F50" s="0" t="inlineStr">
+      <c r="E50" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/rive-unlocking-the-power-of-interactive-motion</t>
         </is>
+      </c>
+      <c r="F50" s="0">
+        <v>1</v>
       </c>
       <c r="G50" s="0">
         <v>1000</v>
@@ -10748,13 +10730,13 @@
           <t>Discusses circularity and how sustainable reuse can shape the future of mobility at Cars24.</t>
         </is>
       </c>
-      <c r="E51" s="0">
-        <v>1</v>
-      </c>
-      <c r="F51" s="0" t="inlineStr">
+      <c r="E51" s="0" t="inlineStr">
         <is>
           <t>https://autonauts.cars24.com/blog/circularity-pioneering-the-future-of-mobility-with-cars24</t>
         </is>
+      </c>
+      <c r="F51" s="0">
+        <v>1</v>
       </c>
       <c r="G51" s="0">
         <v>1000</v>
@@ -10923,7 +10905,7 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>Slides per post</t>
+          <t>URL</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
@@ -10933,24 +10915,24 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>Number of images for this row. 1 = single image; 2-10 = carousel slides for this post.</t>
+          <t>Canonical article or destination URL.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>URL</t>
+          <t>Number of slides</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>Canonical article or destination URL.</t>
+          <t>Defaults to 1. Use 2-5 for carousel rows; above 5 should be intentionally confirmed before generation.</t>
         </is>
       </c>
     </row>
@@ -11244,7 +11226,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C23"/>
+  <autoFilter ref="A1:C24"/>
 </worksheet>
 </file>
 
@@ -11292,7 +11274,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>SlidesPerPost</t>
+          <t>SlideCounts</t>
         </is>
       </c>
     </row>
@@ -11332,10 +11314,8 @@
           <t>Headline-left + system-right</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="H2" s="0">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -11374,10 +11354,8 @@
           <t>Headline-left + flow-right</t>
         </is>
       </c>
-      <c r="H3" s="0" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="H3" s="0">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -11416,10 +11394,8 @@
           <t>Centre workflow</t>
         </is>
       </c>
-      <c r="H4" s="0" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="H4" s="0">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -11446,10 +11422,8 @@
           <t>Headline-left + hero-right</t>
         </is>
       </c>
-      <c r="H5" s="0" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="H5" s="0">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -11468,10 +11442,8 @@
           <t>Centre lockup</t>
         </is>
       </c>
-      <c r="H6" s="0" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="H6" s="0">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -11486,10 +11458,8 @@
           <t>Data-led split</t>
         </is>
       </c>
-      <c r="H7" s="0" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="H7" s="0">
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -11504,10 +11474,8 @@
           <t>Three-figure hero</t>
         </is>
       </c>
-      <c r="H8" s="0" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="H8" s="0">
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -11522,10 +11490,8 @@
           <t>Product-builder scene</t>
         </is>
       </c>
-      <c r="H9" s="0" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="H9" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -11540,10 +11506,8 @@
           <t>Dashboard-to-action</t>
         </is>
       </c>
-      <c r="H10" s="0" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="H10" s="0">
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -11558,10 +11522,8 @@
           <t>Restrained centre</t>
         </is>
       </c>
-      <c r="H11" s="0" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="H11" s="0">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -11587,7 +11549,7 @@
       <c r="F13" s="0"/>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>No-text balanced hero</t>
+          <t>Map/chain layout</t>
         </is>
       </c>
       <c r="H13" s="0"/>
@@ -11601,7 +11563,7 @@
       <c r="F14" s="0"/>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>Map/chain layout</t>
+          <t>Roadmap arc</t>
         </is>
       </c>
       <c r="H14" s="0"/>
@@ -11615,7 +11577,7 @@
       <c r="F15" s="0"/>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>Roadmap arc</t>
+          <t>Showroom hero</t>
         </is>
       </c>
       <c r="H15" s="0"/>
@@ -11629,7 +11591,7 @@
       <c r="F16" s="0"/>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>Showroom hero</t>
+          <t>Metaphor-led</t>
         </is>
       </c>
       <c r="H16" s="0"/>
@@ -11643,7 +11605,7 @@
       <c r="F17" s="0"/>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>Metaphor-led</t>
+          <t>Portrait-right</t>
         </is>
       </c>
       <c r="H17" s="0"/>
@@ -11657,7 +11619,7 @@
       <c r="F18" s="0"/>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>Portrait-right</t>
+          <t>Car cutaway</t>
         </is>
       </c>
       <c r="H18" s="0"/>
@@ -11671,7 +11633,7 @@
       <c r="F19" s="0"/>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>Car cutaway</t>
+          <t>People-led hero</t>
         </is>
       </c>
       <c r="H19" s="0"/>
@@ -11685,7 +11647,7 @@
       <c r="F20" s="0"/>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>People-led hero</t>
+          <t>Product promise</t>
         </is>
       </c>
       <c r="H20" s="0"/>
@@ -11699,7 +11661,7 @@
       <c r="F21" s="0"/>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>Product promise</t>
+          <t>Metaphor portrait</t>
         </is>
       </c>
       <c r="H21" s="0"/>
@@ -11713,7 +11675,7 @@
       <c r="F22" s="0"/>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>Metaphor portrait</t>
+          <t>Minimal title-led</t>
         </is>
       </c>
       <c r="H22" s="0"/>
@@ -11727,7 +11689,7 @@
       <c r="F23" s="0"/>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>Minimal title-led</t>
+          <t>Flowing system</t>
         </is>
       </c>
       <c r="H23" s="0"/>
@@ -11741,7 +11703,7 @@
       <c r="F24" s="0"/>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>Flowing system</t>
+          <t>Timeline</t>
         </is>
       </c>
       <c r="H24" s="0"/>
@@ -11755,7 +11717,7 @@
       <c r="F25" s="0"/>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>Timeline</t>
+          <t>Architecture diagram</t>
         </is>
       </c>
       <c r="H25" s="0"/>
@@ -11769,7 +11731,7 @@
       <c r="F26" s="0"/>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>Architecture diagram</t>
+          <t>Confusion-to-clarity path</t>
         </is>
       </c>
       <c r="H26" s="0"/>
@@ -11783,7 +11745,7 @@
       <c r="F27" s="0"/>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>Confusion-to-clarity path</t>
+          <t>Waveform guardrail</t>
         </is>
       </c>
       <c r="H27" s="0"/>
@@ -11797,7 +11759,7 @@
       <c r="F28" s="0"/>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>Waveform guardrail</t>
+          <t>Headline-dominant</t>
         </is>
       </c>
       <c r="H28" s="0"/>
@@ -11811,7 +11773,7 @@
       <c r="F29" s="0"/>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>Headline-dominant</t>
+          <t>Ownership system</t>
         </is>
       </c>
       <c r="H29" s="0"/>
@@ -11825,7 +11787,7 @@
       <c r="F30" s="0"/>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>Ownership system</t>
+          <t>Centre horizon</t>
         </is>
       </c>
       <c r="H30" s="0"/>
@@ -11839,7 +11801,7 @@
       <c r="F31" s="0"/>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>Centre horizon</t>
+          <t>Reflective split</t>
         </is>
       </c>
       <c r="H31" s="0"/>
@@ -11853,7 +11815,7 @@
       <c r="F32" s="0"/>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>Reflective split</t>
+          <t>Calm checklist</t>
         </is>
       </c>
       <c r="H32" s="0"/>
@@ -11867,7 +11829,7 @@
       <c r="F33" s="0"/>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>Calm checklist</t>
+          <t>Patterned life/work rhythm</t>
         </is>
       </c>
       <c r="H33" s="0"/>
@@ -11881,7 +11843,7 @@
       <c r="F34" s="0"/>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>Patterned life/work rhythm</t>
+          <t>Process path</t>
         </is>
       </c>
       <c r="H34" s="0"/>
@@ -11895,7 +11857,7 @@
       <c r="F35" s="0"/>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>Process path</t>
+          <t>Loop-to-output</t>
         </is>
       </c>
       <c r="H35" s="0"/>
@@ -11909,7 +11871,7 @@
       <c r="F36" s="0"/>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>Loop-to-output</t>
+          <t>Minimal repeated form</t>
         </is>
       </c>
       <c r="H36" s="0"/>
@@ -11923,7 +11885,7 @@
       <c r="F37" s="0"/>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>Minimal repeated form</t>
+          <t>Road-risk scene</t>
         </is>
       </c>
       <c r="H37" s="0"/>
@@ -11937,7 +11899,7 @@
       <c r="F38" s="0"/>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>Road-risk scene</t>
+          <t>Rating hierarchy</t>
         </is>
       </c>
       <c r="H38" s="0"/>
@@ -11951,7 +11913,7 @@
       <c r="F39" s="0"/>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>Rating hierarchy</t>
+          <t>Portrait + trail</t>
         </is>
       </c>
       <c r="H39" s="0"/>
@@ -11965,7 +11927,7 @@
       <c r="F40" s="0"/>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>Portrait + trail</t>
+          <t>Workflow system</t>
         </is>
       </c>
       <c r="H40" s="0"/>
@@ -11979,7 +11941,7 @@
       <c r="F41" s="0"/>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>Workflow system</t>
+          <t>Product-tech card</t>
         </is>
       </c>
       <c r="H41" s="0"/>
@@ -11993,7 +11955,7 @@
       <c r="F42" s="0"/>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>Product-tech card</t>
+          <t>Recommendation paths</t>
         </is>
       </c>
       <c r="H42" s="0"/>
@@ -12007,7 +11969,7 @@
       <c r="F43" s="0"/>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>Recommendation paths</t>
+          <t>Calm people hero</t>
         </is>
       </c>
       <c r="H43" s="0"/>
@@ -12021,7 +11983,7 @@
       <c r="F44" s="0"/>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>Calm people hero</t>
+          <t>Docs-to-data</t>
         </is>
       </c>
       <c r="H44" s="0"/>
@@ -12035,7 +11997,7 @@
       <c r="F45" s="0"/>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>Docs-to-data</t>
+          <t>Signal stream</t>
         </is>
       </c>
       <c r="H45" s="0"/>
@@ -12049,7 +12011,7 @@
       <c r="F46" s="0"/>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>Signal stream</t>
+          <t>Voice intelligence</t>
         </is>
       </c>
       <c r="H46" s="0"/>
@@ -12063,7 +12025,7 @@
       <c r="F47" s="0"/>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>Voice intelligence</t>
+          <t>Timeline portrait</t>
         </is>
       </c>
       <c r="H47" s="0"/>
@@ -12077,7 +12039,7 @@
       <c r="F48" s="0"/>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>Timeline portrait</t>
+          <t>Motion interface</t>
         </is>
       </c>
       <c r="H48" s="0"/>
@@ -12091,24 +12053,10 @@
       <c r="F49" s="0"/>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>Motion interface</t>
+          <t>Circular system</t>
         </is>
       </c>
       <c r="H49" s="0"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="0"/>
-      <c r="B50" s="0"/>
-      <c r="C50" s="0"/>
-      <c r="D50" s="0"/>
-      <c r="E50" s="0"/>
-      <c r="F50" s="0"/>
-      <c r="G50" s="0" t="inlineStr">
-        <is>
-          <t>Circular system</t>
-        </is>
-      </c>
-      <c r="H50" s="0"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>

</xml_diff>